<commit_message>
feat(discovery): universalize Windows File Explorer discovery hub and [C-81] invariant across fleet
</commit_message>
<xml_diff>
--- a/مكتبة الأوامر.xlsx
+++ b/مكتبة الأوامر.xlsx
@@ -4808,7 +4808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="29" min="1" max="1"/>
@@ -5603,6 +5603,52 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="45" customHeight="1" s="55">
+      <c r="A36" s="67" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="68" t="inlineStr">
+        <is>
+          <t>⚡ التوجيه الإلزامي لـ Claude لتشغيل عمال GLM 5.3 Flash بالتوازي (Multi-Worker Parallel Dispatch)</t>
+        </is>
+      </c>
+      <c r="C36" s="69" t="inlineStr">
+        <is>
+          <t>Act as Master Orchestrator (Claude Opus Max). You are commanded to actively dispatch two or more GLM 5.3 Flash workers in parallel across non-colliding scopes:
+1. Worker A (OpenCode CLI): &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_A_prompt}"
+2. Worker B (Cline CLI / Parallel OpenCode): &amp; cline "{task_B_prompt}" OR &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_B_prompt}"
+Decompose independent sub-tasks, launch workers simultaneously in background, enforce disjoint file paths, and retain exclusive authority for architecture reviews and test approvals [APPROVED].</t>
+        </is>
+      </c>
+      <c r="D36" s="70" t="inlineStr">
+        <is>
+          <t>توجيه قيادي صارم يلزم Claude Code CLI (Opus Max) بتفكيك المهام البرمجية وتشغيل 2 إلى 4 عمال من نموذج GLM 5.3 Flash بالتوازي عبر OpenCode CLI و Cline CLI على مسارات ملفات غير متصادمة، مما يعظم سرعة الإنجاز بنسبة 300%+ ويحفظ ميزانية توكنز كلود للمراجعات المعمارية واحتكار الاختبارات حصرياً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1" s="55">
+      <c r="A37" s="67" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="68" t="inlineStr">
+        <is>
+          <t>⚡ التوجيه الإلزامي لـ Claude لتشغيل عمال GLM 5.3 Flash بالتوازي (Multi-Worker Parallel Dispatch)</t>
+        </is>
+      </c>
+      <c r="C37" s="69" t="inlineStr">
+        <is>
+          <t>Act as Master Orchestrator (Claude Opus Max). You are commanded to actively dispatch two or more GLM 5.3 Flash workers in parallel across non-colliding scopes:
+1. Worker A (OpenCode CLI): &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_A_prompt}"
+2. Worker B (Cline CLI / Parallel OpenCode): &amp; cline "{task_B_prompt}" OR &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_B_prompt}"
+Decompose independent sub-tasks, launch workers simultaneously in background, enforce disjoint file paths, and retain exclusive authority for architecture reviews and test approvals [APPROVED].</t>
+        </is>
+      </c>
+      <c r="D37" s="70" t="inlineStr">
+        <is>
+          <t>توجيه قيادي صارم يلزم Claude Code CLI (Opus Max) بتفكيك المهام البرمجية وتشغيل 2 إلى 4 عمال من نموذج GLM 5.3 Flash بالتوازي عبر OpenCode CLI و Cline CLI على مسارات ملفات غير متصادمة، مما يعظم سرعة الإنجاز بنسبة 300%+ ويحفظ ميزانية توكنز كلود للمراجعات المعمارية واحتكار الاختبارات حصرياً.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3"/>
@@ -5615,7 +5661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6003,6 +6049,26 @@
       <c r="D17" s="70" t="inlineStr">
         <is>
           <t>وكيل المتابعة المستمرة (babysit-pr): حصاد كافة ملاحظات المراجعين على الـ PR، التحقق منها على الكود الحي، إصلاح المشاكل الحقيقية، والرد في الخيوط وإعادة الفحص حتى الدمج.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="55">
+      <c r="A18" s="67" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="68" t="inlineStr">
+        <is>
+          <t>🌊 توجيه الموجة المعمارية المستقلة والتوزيع المتوازي للأسطول (Google Stitch &amp; Operations Control)</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t># 🌊 AUTONOMOUS WAVE EXECUTION &amp; MULTI-AGENT PARALLEL DIRECTIVE\n\nTarget: Claude Code CLI (Opus Max — Master Orchestrator &amp; Sole Testing Monopoly)\nParallel Workers: OpenCode CLI (GLM 5.3 Flash), Cline CLI, Antigravity CLI (agcli)\nDesign Paradigm: Google Stitch &amp; Dribbble Operations Control (Micro-Sparklines, Icon Navigation Rail, Outcomes Matrix)\nWorkspace: f:\AI PROJECTS\Claude+Antigravity -production\taj_al_waqar_global\n\nExecution Protocol:\n1. Analyze: Inspect newly authored code under lib/ for clean static analysis.\n2. Author Tests: Comprehensive unit and widget tests under test/ for all domain contracts &amp; widgets.\n3. Execute Verification Suite: C:\flutter_sdk\bin\flutter test --concurrency=1 (0 failures, 0 regressions).\n4. Certification: Inscribe formal ADR in MEMORY_STORE.md and grant [APPROVED TO SHIP] in FLEET_LOG.md.</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="inlineStr">
+        <is>
+          <t>موجه قيادي معتمد لتنفيذ موجات التطوير البرمجي بالأسطول المتوازي، مع الالتزام الصارم بمعايير Google Stitch ولوحات تحكم Dribbble ومونوپولي الاختبارات لكلود كود.</t>
         </is>
       </c>
     </row>
@@ -6387,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6689,6 +6755,26 @@
       <c r="D14" s="70" t="inlineStr">
         <is>
           <t>تفعيل مهارة وجسر أبحاث Duck.ai للاستعلام المجاني من نماذج GPT-4o-mini و Claude 3 Haiku و Llama 3.3 وتوفير Sandbox لاختبارات n8n و FastMCP وحفظ كوتا النماذج التجارية لوكالة Autovem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1" s="55">
+      <c r="A15" s="67" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="68" t="inlineStr">
+        <is>
+          <t>🎬 أخصائي المونتاج والإخراج الفني بالذكاء الاصطناعي (ai-video-montage-specialist)</t>
+        </is>
+      </c>
+      <c r="C15" s="69" t="inlineStr">
+        <is>
+          <t>قم بتحليل فيديو العميل [البراند] واستخراج ملف الصوت والـ Contact Sheet، واستخرج التوقيتات الدقيقة بالملي ثانية عبر Whisper، ونفذ القطع الأولي (Rough Cut) بإزالة السكتات وتوليد ملف EDL، ثم طبق نظام التصميم ومكافحة النمطية في تركيبة Remotion.</t>
+        </is>
+      </c>
+      <c r="D15" s="70" t="inlineStr">
+        <is>
+          <t>أخصائي المونتاج والإخراج الفني الذاتي: إدارة خط إنتاج الفيديو البرمجي بالكود استناداً لهندسة غريب الشيخ؛ فحص FFmpeg واستخراج الصوت النقي 16kHz، تحليل المساحات السلبية (Negative Space) لمنع تغطية وجه المتحدث، تفريغ Whisper بالملي ثانية، توليد ملفات EDL لبريمير ودافينشي، إخراج المشاهد بأنماط Focus و Whiteboard و Screencast، ورندرة Remotion React ومكافحة ركاكة الـ AI Slop.</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -7417,6 +7503,28 @@
       <c r="D1" s="71" t="inlineStr">
         <is>
           <t>الوصف والاستخدام (Description &amp; Notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>📂 إظهار الملفات في مستكشف ويندوز وتصديرها لسطح المكتب (Reveal &amp; Desktop Hub - C-81)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>reveal "&lt;Full_Path&gt;"</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>المعيار الإلزامي [C-81] لأدوات ومستندات Antigravity: يقوم بترجمة مسارات WSL إلى ويندوز، نسخ الملف فوراً إلى مجلد المستندات_المولدة على سطح المكتب (C:\Users\Kt\Desktop\المستندات_المولدة\)، وفتح مستكشف الملفات مع تظليل الملف تلقائياً وبشكل غير تزامني.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(prompt-library): restore 11 missing rows, deduplicate, and curate pstack fleet suite & guide (Hook 26 via Hook 31)
</commit_message>
<xml_diff>
--- a/مكتبة الأوامر.xlsx
+++ b/مكتبة الأوامر.xlsx
@@ -48,7 +48,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -211,6 +211,37 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <b val="1"/>
+      <color rgb="00002060"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -256,7 +287,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -515,11 +546,40 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -706,6 +766,40 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4362,7 +4456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="55" min="1" max="1"/>
@@ -4540,12 +4634,171 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="21" customHeight="1" s="55"/>
-    <row r="10" ht="84" customHeight="1" s="55"/>
-    <row r="11" ht="21" customHeight="1" s="55"/>
-    <row r="12" ht="21" customHeight="1" s="55"/>
-    <row r="13" ht="21" customHeight="1" s="55"/>
-    <row r="14" ht="42" customHeight="1" s="55"/>
+    <row r="9" ht="45" customHeight="1" s="55">
+      <c r="A9" s="67" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="68" t="inlineStr">
+        <is>
+          <t>🎨 تصميم شعار أوتوفيم إيجنسي (Autovem Logo)</t>
+        </is>
+      </c>
+      <c r="C9" s="69" t="inlineStr">
+        <is>
+          <t>Minimalist corporate vector logo for tech agency Autovem. Flat geometric emblem fusing letter A with upward growth arrow and cybernetic loop. Colors: electric cyan and neon violet gradient on solid obsidian background #0a0a14. Clean typography Autovem, modern tech brand identity, crisp vector art.</t>
+        </is>
+      </c>
+      <c r="D9" s="70" t="inlineStr">
+        <is>
+          <t>برومبت مهندس لتصميم هوية وشعار وكالة Autovem يجمع بين ركائز النمو والذكاء الاصطناعي وهندسة البرمجيات.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="55">
+      <c r="A10" s="67" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="68" t="inlineStr">
+        <is>
+          <t>🏛️ توليد Brand System Design كامل من الصفر (Brand Discovery → Brand Book)</t>
+        </is>
+      </c>
+      <c r="C10" s="69" t="inlineStr">
+        <is>
+          <t>قم بتفعيل جلسة Grill-Me لبناء Brand System Design متكامل:
+1. اسأل عن: اسم البراند، طبيعة العمل، الشخصية (warm/bold/trusted)، الجمهور، الموقع الجغرافي، الألوان المتوفرة (HEX)، اللوجو (مسار الملف)، أماكن التطبيق (Web/App/Print/Social)، لغة الـ Wordmark، أسلوب الصور المطلوب.
+2. بعد الإجابات: ولّد Color Palette مع CSS Custom Properties، منظومة خطوط Cairo+Tajawal+Inter، Logo Usage Guidelines مع Clear Zone، أسلوب التصوير (Do/Don't)، Design Tokens جاهزة للمطورين، وقواعد التطبيق على (Website / Proposals / Social Media / Business Cards).
+3. سلّم الوثيقة النهائية كـ Markdown + CSS Variables جاهزة للمصمم والمطور.</t>
+        </is>
+      </c>
+      <c r="D10" s="70" t="inlineStr">
+        <is>
+          <t>بروتوكول متكامل لبناء هوية بصرية احترافية عبر جلسة استكشاف تفاعلية (Grill-Me) تشمل الألوان والخطوط واللوجو والصور وتوكنز CSS للمطورين.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1" s="55">
+      <c r="A11" s="67" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="68" t="inlineStr">
+        <is>
+          <t>📊 هندسة لوحة تحليلات الحاويات والمبيعات الشهرية متعددة الوسائط (Multimodal Fleet Analytics &amp; Excel Importer)</t>
+        </is>
+      </c>
+      <c r="C11" s="69" t="inlineStr">
+        <is>
+          <t>قم ببناء وترقية لوحة تحليلات تفاعلية شاملة لمبيعات وإيجارات أسطول الحاويات (HTML/CSS/JS Offline Standalone) مع دمج محرك استيراد Excel/CSV ومواءمة المتطلبات التشغيلية التالية:
+1. استخراج وتدقيق البيانات من كشف المبيعات (PDF / Excel): مطابقة صافي المبيعات، ضريبة القيمة المضافة 15%، والإجمالي الشامل بدقة الهللة، وربطها برقم الحاوية، رقم السيارة، والسائق.
+2. تحليل المقاسات الثلاثة (12، 20، 30 ياردة): حساب عدد الردود لكل مقاس ونسبتها المئوية من الإجمالي، مع صافي الإيراد ومتوسط سعر الرد لكل مقاس.
+3. الترتيب التنازلي للعملاء: جدول ورسم بياني تفاعلي يرتب كافة العملاء تنازلياً حسب عدد الردود وإجمالي المبالغ ومتوسط سعر الرد.
+4. حصر السائقين وحساب العمولات: حساب إجمالي عدد ردود كل سائق ومستحقاته المالية آلياً بواقع عمولة 10 ريال لكل رد منجز.
+5. إنتاجية أسطول السيارات: حساب متوسط عدد الردود اليومية لكل سيارة/شاحنة على أساس 26 يوم عمل شهرياً (الردود ÷ 26)، مع مؤشر الإنتاجية الكلية للأسطول.
+6. محرك استيراد Excel/CSV التفاعلي: زر استيراد مباشر مدعوم بـ SheetJS محلياً لقراءة ملفات .xlsx و .csv وتطبيع المقاسات والأحياء تلقائياً وتحديث كافة الرسوم البيانية والجداول والـ KPIs لحظياً دون الحاجة لإعادة تحميل الصفحة.
+7. الالتزام بمعايير الأرقام الإنجليزية (0-9) والهوية البصرية الداكنة المتناسقة مع تجربة مستخدم سريعة وكاملة دون اتصال بالإنترنت.</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>برومبت مهندس وشامل لبناء وترقية لوحات تحليلات الحاويات وإدارة أساطيل النقل من كشوفات الـ PDF والإكسيل الشهرية، يشمل استخراج وتدقيق الردود، توزيع المقاسات (12، 20، 30 ياردة)، الإيرادات الصافية والشاملة للضريبة، ترتيب العملاء تنازلياً، حساب عمولات السائقين (10 ريال/رد)، متوسط إنتاجية الشاحنات لـ 26 يوم عمل، مع محرك استيراد Excel/CSV مباشر وتحديث لحظي دون اتصال.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1" s="55">
+      <c r="A12" s="67" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="68" t="inlineStr">
+        <is>
+          <t>📦 تجهيز وتطهير لوحة تحليلات شجن للتسليم للعميل وتفعيل محرك الاستيراد بالذكاء الاصطناعي المجاني (Client Ready &amp; Free AI Vision)</t>
+        </is>
+      </c>
+      <c r="C12" s="69" t="inlineStr">
+        <is>
+          <t>قم بتجهيز وتطهير لوحة تحليلات واستهلاك حاويات شجن (لوحة_استهلاك_عملاء_حاويات_شجن.html) للتسليم النهائي المباشر للعميل، وتفعيل منظومة الاستيراد الذكي المجانية وفق المعايير التالية:
+1. حزمة التسليم الذاتية والاستقلالية (Standalone &amp; Zero Breakage):
+   - دعم التحميل الهجين الذكي للمكتبات (CDN Fallback): تأكد أن ملفات SheetJS (xlsx.full.min.js) و PDF.js (pdf.min.js) يتم استدعاؤها محلياً أولاً، وفي حال فتح العميل للملف كملف HTML منفرد بدون الملفات المجاورة، يتم التراجع تلقائياً وسلساً لجلب المكتبات من شبكات CDN موثوقة (cdnjs/jsdelivr) لضمان عدم توقف الاستيراد إطلاقاً.
+   - التحقق من تضمين محرك الرسوم البيانية Chart.js داخلياً (Inlined) والخطوط الرسمية (Noto Kufi Arabic &amp; JetBrains Mono) لتوفير أداء فائق ومظهر متناسق.
+2. التطهير والتدقيق الشامل للواجهة (UI &amp; Code Sanitization):
+   - إزالة أي متبقيات لتعليقات التطوير البرمجية أو إشارات المتطلبات الداخلية والرموز الاختبارية.
+   - مراجعة هوية شجن البصرية الفاخرة (Dark Logistics Theme: ألوان الكانفاس الداكن #0c0e14، التوهج الكهرماني اللوجستي #f59e0b، والأخضر التنفيذي #10b981).
+   - التحقق من تفعيل الترقيم الإنجليزي القياسي (0-9) لكافة الأرقام، وتنسيق العملات (ر.س) والتواريخ والنسب المئوية.
+3. تفعيل ودعم محرك الاستيراد بالذكاء الاصطناعي المجاني (Free AI Vision Integration):
+   - توضيح المسار المباشر (On-Device Local Parser): تدريب العميل على أن كشوفات الـ PDF الرسمية ومصنفات الإكسيل الأصلية لا تتطلب أي مفتاح API وتعمل مجاناً وبسرعة البرق محلياً.
+   - إعداد ودعم بوابة Google Gemini Multimodal Vision API المجانية 100% عبر Google AI Studio للفواتير المصورة ضوئياً (OCR) وكشوفات السكانر.
+   - تضمين دليل إرشادي مبسط خطوة بخطوة للعميل يوضح كيفية إنشاء مفتاح مجاني دائم خلال 30 ثانية من aistudio.google.com/app/apikey ولصقه في نافذة الاستيراد وحفظه في ذاكرة المتصفح الآمنة (localStorage).
+   - توفير مفتاح تجريبي آمن مسبق الإعداد أو خيار التفعيل الفوري للمعاينة والتسليم السلس.
+4. حزمة التسليم النهائية (Client Handover Package):
+   - تجهيز ملف مضغوط ZIP يحتوي على: ملف اللوحة المكتمل والمطهر، المكتبات المحلية المساعدة، ونموذج كشف المبيعات المعتمد، مع دليل استخدام سريع موجه لمدير العمليات بشركة شجن.</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="inlineStr">
+        <is>
+          <t>برومبت هندسي شامل لتجهيز وتطهير لوحة تحليلات حاويات شجن للتسليم النهائي للعميل، يتضمن تطبيق التحميل الاحتياطي الهجين للمكتبات (CDN Fallback) لضمان العمل المنفرد، وتطهير الواجهة من أي آثار تطوير داخلية، ودمج وتفعيل بوابات الذكاء الاصطناعي المجانية (Google Gemini Vision API عبر Google AI Studio) للفواتير المصورة، مع صياغة دليل إرشادي سريع للتسليم والتشغيل المباشر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1" s="55">
+      <c r="A13" s="67" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="68" t="inlineStr">
+        <is>
+          <t>🛠️ إصلاح وتأمين محرك استيراد كشوف مبيعات PDF في لوحة تحكم شجن</t>
+        </is>
+      </c>
+      <c r="C13" s="69" t="inlineStr">
+        <is>
+          <t>قم بتشخيص وحل مشكلة توقف وفشل استيراد كشف مبيعات الـ PDF (السنوي والشهري) في لوحة تحكم شجن: فحص مسارات ملفات pdf.min.js و pdf.worker.js في المجلدات الفرعية، وتأمين بيئة file:// بتحميل الـ Worker في الخيط الرئيسي لمنع قيود CORS، وإعادة تعيين قيمة input[type=file] لمنع تجميد إعادة الاختيار، وضمان التدقيق الحسابي للضريبة والمطابقة التامة للمجاميع.</t>
+        </is>
+      </c>
+      <c r="D13" s="70" t="inlineStr">
+        <is>
+          <t>موجه هندسي تخصصي لإصلاح وتأمين محركات استيراد ملفات الـ PDF في لوحات بيانات SPAs المحلية على بيئات المتصفح، معالجة قيود Web Workers و CORS على بروتوكول file://، والتدقيق الحسابي التلقائي للبيانات المستخرجة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" s="55">
+      <c r="A14" s="75" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="76" t="inlineStr">
+        <is>
+          <t>🔬 فحص وتدقيق الأسطول لمطابقة البيانات والرسوم البيانية (Excel vs PDF vs Dashboard Audit)</t>
+        </is>
+      </c>
+      <c r="C14" s="77" t="inlineStr">
+        <is>
+          <t>You are the Master Orchestrator and Staff Architect (Claude Code CLI - Opus 5.5 High) leading the full multi-worker fleet (Workers A, B, C, D, and Codex) as defined in fleet_config.json.
+Your mission is to perform an exhaustive, multi-dimensional test and mathematical reconciliation comparing the Shajan Containers Interactive Dashboard (Clients/01_Shajan_Containers/لوحة_استهلاك_عملاء_حاويات_شجن.html) against:
+1. The Excel ledger (Clients/01_Shajan_Containers/تقرير الإيجارات من 01 01 حتى 26 09 2026.xlsx)
+2. The 18-page certified PDF statement (Clients/01_Shajan_Containers/تقرير الإيجارات من 01 01 حتى 30 09 2026.pdf)
+TEST &amp; RECONCILIATION WORKSTREAMS:
+1. SCOPE &amp; TIMEFRAME RECONCILIATION (Worker B - Muse Spark 1.3 &amp; Codex GPT-5.6):
+   - Baseline Scope Check: Excel covers 01-01-2026 to 26-09-2026 (929 rows). PDF covers the full month up to 30-09-2026 (957 rows).
+   - Apple-to-Apple Window (01-01 to 26-09): Reconcile the exact 6 delta rows between Excel (929 rows) and Dashboard (923 rows).
+   - In Full Month (to 30/09): Verify all 957 PDF rows parse with 100% fidelity.
+2. FINANCIAL &amp; VAT CONSISTENCY AUDIT (Worker B - Muse Spark 1.3):
+   - Verify: Gross = Net + VAT across every row and aggregated KPIs.
+   - For 18-page PDF: Verify Gross is 486,017.50 SAR with explicit VAT accumulation of 31,175.11 SAR.
+   - For Excel: Verify Gross is 510,296.65 SAR (Net 468,568.48 + VAT 41,728.17 SAR).
+3. CONTAINER SIZES &amp; CLIENT RANKING RECONCILIATION (Worker D - agcli):
+   - Proportional Sizes: Verify 20-yard dominance (~89%), 12-yard (~8%), and 30-yard (~3%) align across Excel, PDF, and Chart.js.
+   - Top Clients Ranking: Verify identical order: 1st Belda, 2nd GIO, 3rd Abu Tamim, 4th Tawajud, 5th Abaad.
+4. STRICT FRIDAY EXCLUSION INVARIANT:
+   - FRIDAY IS NEVER COUNTED AS A WORKING DAY under any circumstances.
+   - getWorkingDays() must strictly omit Fridays (cur.getDay() === 5).
+   - Verify September 2026 working days equals exactly 26 days (30 calendar days minus 4 Fridays).
+EXCLUSIVE TESTING MONOPOLY &amp; QUALITY GATE:
+As Claude Code CLI, execute automated headless assertions, compare values programmatically, inspect visual chart rendering, and grant the final [APPROVED] verdict once zero discrepancies remain.</t>
+        </is>
+      </c>
+      <c r="D14" s="78" t="inlineStr">
+        <is>
+          <t>برومبت مهندس لقيادة أسطول الـ CLIs بالكامل لإجراء فحص وتدقيق رياضي وبصري دقيق للوحة تحليلات شجن ومقارنة أرقام ورسوم ملف الإكسيل مع ملف الـ PDF لنفس البيانات والتحقق من استبعاد يوم الجمعة.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" paperSize="3"/>
@@ -4808,7 +5061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="29" min="1" max="1"/>
@@ -4841,436 +5094,457 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="31.95" customHeight="1" s="55">
-      <c r="A2" s="31" t="n">
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="28" t="inlineStr">
+      <c r="B2" s="68" t="inlineStr">
         <is>
           <t>المساعدة وعرض الأوامر</t>
         </is>
       </c>
-      <c r="C2" s="30" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>/help</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="70" t="inlineStr">
         <is>
           <t>يعرض قائمة بجميع الأوامر المتاحة وتلميحات الاستخدام داخل الجلسة.</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.95" customHeight="1" s="55">
-      <c r="A3" s="31" t="n">
+      <c r="E2" s="83" t="n"/>
+    </row>
+    <row r="3" ht="45" customHeight="1" s="55">
+      <c r="A3" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>بدء محادثة جديدة نظيفة</t>
         </is>
       </c>
-      <c r="C3" s="30" t="inlineStr">
+      <c r="C3" s="69" t="inlineStr">
         <is>
           <t>/clear</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="70" t="inlineStr">
         <is>
           <t>إعادة ضبط المحادثة وسياق الذاكرة مع بقاء تعليمات وقواعد CLAUDE.md نشطة.</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="31.95" customHeight="1" s="55">
-      <c r="A4" s="31" t="n">
+      <c r="E3" s="83" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="55">
+      <c r="A4" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>ضغط سياق المحادثة</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>/compact</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>تلخيص المحادثة لتقليل استهلاك التوكنز والذاكرة، مع إمكانية تحديد محور التركيز مثل /compact focus on auth.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="31.95" customHeight="1" s="55">
-      <c r="A5" s="31" t="n">
+      <c r="E4" s="83" t="n"/>
+    </row>
+    <row r="5" ht="45" customHeight="1" s="55">
+      <c r="A5" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>عرض استهلاك السياق التفاعلي</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="69" t="inlineStr">
         <is>
           <t>/context</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>عرض رسم بياني يوضح استهلاك نافذة السياق وتوزيع التوكنز بين الملفات والمحادثة.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="31.95" customHeight="1" s="55">
-      <c r="A6" s="31" t="n">
+      <c r="E5" s="83" t="n"/>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="55">
+      <c r="A6" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>مستعرض الفروقات البرمجية</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="69" t="inlineStr">
         <is>
           <t>/diff</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>فتح عارض تفاعلي لفحص التغييرات والتعديلات غير المحفوظة في الكود.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="31.95" customHeight="1" s="55">
-      <c r="A7" s="31" t="n">
+      <c r="E6" s="83" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="55">
+      <c r="A7" s="67" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>تبديل نموذج الذكاء الاصطناعي</t>
         </is>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="69" t="inlineStr">
         <is>
           <t>/model</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>التبديل بين Sonnet و Opus و Haiku أثناء تشغيل الجلسة مع إمكانية كتابة /model sonnet مباشرة.</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="31.95" customHeight="1" s="55">
-      <c r="A8" s="31" t="n">
+      <c r="E7" s="83" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1" s="55">
+      <c r="A8" s="67" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>حساب التكلفة والتوكنز</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>/cost</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>عرض إجمالي التوكنز المستهلكة في الجلسة والتكلفة المالية المقدرة.</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="31.95" customHeight="1" s="55">
-      <c r="A9" s="31" t="n">
+      <c r="E8" s="83" t="n"/>
+    </row>
+    <row r="9" ht="45" customHeight="1" s="55">
+      <c r="A9" s="67" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="68" t="inlineStr">
         <is>
           <t>عرض حالة وحساب الجلسة</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="69" t="inlineStr">
         <is>
           <t>/status</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>عرض رقم الإصدار الحالي، النموذج النشط، وحالة الحساب والمنظمة.</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="31.95" customHeight="1" s="55">
-      <c r="A10" s="31" t="n">
+      <c r="E9" s="83" t="n"/>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="55">
+      <c r="A10" s="67" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>فحص وتشخيص البيئة</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="69" t="inlineStr">
         <is>
           <t>/doctor</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>فحص صحة اتصال الـ CLI، صلاحيات الملفات، وحالة خوادم MCP والأدوات.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="31.95" customHeight="1" s="55">
-      <c r="A11" s="31" t="n">
+      <c r="E10" s="83" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1" s="55">
+      <c r="A11" s="67" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="68" t="inlineStr">
         <is>
           <t>مراجعة وتدقيق التغييرات</t>
         </is>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="69" t="inlineStr">
         <is>
           <t>/review</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="70" t="inlineStr">
         <is>
           <t>فحص شامل للتعديلات الأخيرة في الفرع الحالي ومقارنتها بمعايير الكود النظيف.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="31.95" customHeight="1" s="55">
-      <c r="A12" s="31" t="n">
+      <c r="E11" s="83" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1" s="55">
+      <c r="A12" s="67" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="68" t="inlineStr">
         <is>
           <t>تعديل ذاكرة المشروع</t>
         </is>
       </c>
-      <c r="C12" s="30" t="inlineStr">
+      <c r="C12" s="69" t="inlineStr">
         <is>
           <t>/memory</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>فتح وإدارة ملفات الذاكرة والقواعد CLAUDE.md المطبقة محلياً وعالمياً.</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="31.95" customHeight="1" s="55">
-      <c r="A13" s="31" t="n">
+      <c r="E12" s="83" t="n"/>
+    </row>
+    <row r="13" ht="45" customHeight="1" s="55">
+      <c r="A13" s="67" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="68" t="inlineStr">
         <is>
           <t>تهيئة مستودع جديد</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="69" t="inlineStr">
         <is>
           <t>/init</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="70" t="inlineStr">
         <is>
           <t>مسح وتحليل بنية المشروع وتوليد ملف CLAUDE.md تلقائياً.</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="31.95" customHeight="1" s="55">
-      <c r="A14" s="31" t="n">
+      <c r="E13" s="83" t="n"/>
+    </row>
+    <row r="14" ht="45" customHeight="1" s="55">
+      <c r="A14" s="67" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="68" t="inlineStr">
         <is>
           <t>سؤال جانبي سريع</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="C14" s="69" t="inlineStr">
         <is>
           <t>/btw [سؤالك]</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="70" t="inlineStr">
         <is>
           <t>طرح استفسار أو سؤال جانبي دون مقاطعة المهمة أو الكود الجاري تنفيذه.</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="31.95" customHeight="1" s="55">
-      <c r="A15" s="31" t="n">
+      <c r="E14" s="83" t="n"/>
+    </row>
+    <row r="15" ht="45" customHeight="1" s="55">
+      <c r="A15" s="67" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="68" t="inlineStr">
         <is>
           <t>الإبلاغ عن خطأ وملاحظة</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
+      <c r="C15" s="69" t="inlineStr">
         <is>
           <t>/bug</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="70" t="inlineStr">
         <is>
           <t>إرسال تقرير خطأ أو مشكلة تقنية مصحوباً بسجل الجلسة للمطورين.</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="31.95" customHeight="1" s="55">
-      <c r="A16" s="31" t="n">
+      <c r="E15" s="83" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1" s="55">
+      <c r="A16" s="67" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="68" t="inlineStr">
         <is>
           <t>إدارة إعدادات الأداة</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" s="69" t="inlineStr">
         <is>
           <t>/config</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="70" t="inlineStr">
         <is>
           <t>عرض وتعديل إعدادات التهيئة للأداة ومسارات العمل والأذونات.</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="31.95" customHeight="1" s="55">
-      <c r="A17" s="31" t="n">
+      <c r="E16" s="83" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1" s="55">
+      <c r="A17" s="67" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="68" t="inlineStr">
         <is>
           <t>تسجيل الدخول للحساب</t>
         </is>
       </c>
-      <c r="C17" s="30" t="inlineStr">
+      <c r="C17" s="69" t="inlineStr">
         <is>
           <t>/login</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="70" t="inlineStr">
         <is>
           <t>توثيق وتسجيل الدخول بحساب Anthropic أو تفعيل اشتراك Claude Pro/Team.</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="31.95" customHeight="1" s="55">
-      <c r="A18" s="31" t="n">
+      <c r="E17" s="83" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="55">
+      <c r="A18" s="67" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="68" t="inlineStr">
         <is>
           <t>تسجيل الخروج</t>
         </is>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="C18" s="69" t="inlineStr">
         <is>
           <t>/logout</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="70" t="inlineStr">
         <is>
           <t>إنهاء الجلسة ومسح مفاتيح المصادقة المخزنة محلياً.</t>
         </is>
       </c>
-    </row>
-    <row r="19" ht="31.95" customHeight="1" s="55">
-      <c r="A19" s="31" t="n">
+      <c r="E18" s="83" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1" s="55">
+      <c r="A19" s="67" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="68" t="inlineStr">
         <is>
           <t>تشغيل الوضع غير التفاعلي</t>
         </is>
       </c>
-      <c r="C19" s="30" t="inlineStr">
+      <c r="C19" s="69" t="inlineStr">
         <is>
           <t>claude -p "prompt"</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="70" t="inlineStr">
         <is>
           <t>تمرير برومبت مباشر وتنفيذه من سطر الأوامر دون فتح الجلسة التفاعلية.</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="31.95" customHeight="1" s="55">
-      <c r="A20" s="31" t="n">
+      <c r="E19" s="83" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1" s="55">
+      <c r="A20" s="67" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="68" t="inlineStr">
         <is>
           <t>استئناف الجلسة السابقة</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="C20" s="69" t="inlineStr">
         <is>
           <t>claude --resume</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="70" t="inlineStr">
         <is>
           <t>استعادة الجلسة السابقة ومواصلة العمل من آخر نقطة توقف.</t>
         </is>
       </c>
-    </row>
-    <row r="21" ht="31.95" customHeight="1" s="55">
-      <c r="A21" s="31" t="n">
+      <c r="E20" s="83" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1" s="55">
+      <c r="A21" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="68" t="inlineStr">
         <is>
           <t>تجاوز طلب الأذونات للأتمتة</t>
         </is>
       </c>
-      <c r="C21" s="30" t="inlineStr">
+      <c r="C21" s="69" t="inlineStr">
         <is>
           <t>claude --dangerously-skip-permissions</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="70" t="inlineStr">
         <is>
           <t>تشغيل كلود بنمط الأتمتة الكامل دون طلب تأكيد بشري لكل أمر (يستخدم في البيئات المعزولة).</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="31.95" customHeight="1" s="55">
-      <c r="A22" s="31" t="n">
+      <c r="E21" s="83" t="n"/>
+    </row>
+    <row r="22" ht="45" customHeight="1" s="55">
+      <c r="A22" s="67" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="68" t="inlineStr">
         <is>
           <t xml:space="preserve">طلب تقرير الاسطول </t>
         </is>
       </c>
-      <c r="C22" s="30" t="inlineStr">
+      <c r="C22" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve"> make a report in arabic pdf about waht the fleet done</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="70" t="inlineStr">
         <is>
           <t xml:space="preserve"> fleet report </t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="31.95" customHeight="1" s="55">
-      <c r="A23" s="31" t="n">
+      <c r="E22" s="83" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1" s="55">
+      <c r="A23" s="67" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="68" t="inlineStr">
         <is>
           <t>رومبت التكليف التفاعلي المباشر (لصقه في طرفية Claude Code)</t>
         </is>
       </c>
-      <c r="C23" s="30" t="inlineStr">
+      <c r="C23" s="69" t="inlineStr">
         <is>
           <t># 🌊 AUTONOMOUS WAVE EXECUTION &amp; VERIFICATION DIRECTIVE
 **Target:** Claude Code CLI (Opus Max — Master Orchestrator &amp; Sole Test Authority)
@@ -5284,22 +5558,23 @@
 Please read the active queue file and proceed autonomously!</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="70" t="inlineStr">
         <is>
           <t>الاستخدام: عند رغبتك في إطلاق أو استكمال أي موجة برمجية داخل طرفية كلود.</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="83.40000000000001" customHeight="1" s="55">
-      <c r="A24" s="31" t="n">
+      <c r="E23" s="83" t="n"/>
+    </row>
+    <row r="24" ht="45" customHeight="1" s="55">
+      <c r="A24" s="67" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="28" t="inlineStr">
+      <c r="B24" s="68" t="inlineStr">
         <is>
           <t>2. برومبت تفعيل التشغيل الآلي في الخلفية (إرساله لـ Antigravity):</t>
         </is>
       </c>
-      <c r="C24" s="30" t="inlineStr">
+      <c r="C24" s="69" t="inlineStr">
         <is>
           <t># 🚀 ACTIVATE AUTONOMOUS FLEET BACKGROUND ORCHESTRATION
 Antigravity, please take full autonomous control in the background:
@@ -5310,23 +5585,24 @@
 5. Keep the recurring background monitoring active every 30 minutes until the entire roadmap is completed.</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="70" t="inlineStr">
         <is>
           <t xml:space="preserve">الاستخدام: عندما تريد أن يتولى Antigravity إدارة وتشغيل الأسطول في الخلفية دون أن تفتح أي طرفية.
 </t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="83.40000000000001" customHeight="1" s="55">
-      <c r="A25" s="31" t="n">
+      <c r="E24" s="83" t="n"/>
+    </row>
+    <row r="25" ht="45" customHeight="1" s="55">
+      <c r="A25" s="67" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="28" t="inlineStr">
+      <c r="B25" s="68" t="inlineStr">
         <is>
           <t>🌟 البرومبت الشامل والذاتي العام (Universal Autonomous Fleet Engine Prompt)</t>
         </is>
       </c>
-      <c r="C25" s="30" t="inlineStr">
+      <c r="C25" s="69" t="inlineStr">
         <is>
           <t># ==============================================================================
 # UNIVERSAL AUTONOMOUS FLEET ENGINE (MASTER RECURSIVE DIRECTIVE)
@@ -5367,54 +5643,57 @@
 Begin the autonomous orchestration cycle now.</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D25" s="70" t="inlineStr">
         <is>
           <t>يكتشف الخطوة التالية بنفسه: يقرأ FLEET_LOG.md فيرى أن مهام Track A انتهت، فينتقل تلقائياً لـ Track B ويشغل opencode run، ثم يختبر الكود ويعتمد الموجة ويفتح الموجة التالية فوراً! 🚀</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="30" customHeight="1" s="55">
-      <c r="A26" s="31" t="n">
+      <c r="E25" s="83" t="n"/>
+    </row>
+    <row r="26" ht="45" customHeight="1" s="55">
+      <c r="A26" s="67" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B26" s="68" t="inlineStr">
         <is>
           <t>Push Claude to get ready to make "/clear"</t>
         </is>
       </c>
-      <c r="C26" s="30" t="inlineStr">
+      <c r="C26" s="69" t="inlineStr">
         <is>
           <t>should I make /clear now?</t>
         </is>
       </c>
-      <c r="D26" s="14" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="55">
-      <c r="A27" s="31" t="n">
+      <c r="D26" s="70" t="n"/>
+      <c r="E26" s="83" t="n"/>
+    </row>
+    <row r="27" ht="45" customHeight="1" s="55">
+      <c r="A27" s="67" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="28" t="inlineStr">
+      <c r="B27" s="68" t="inlineStr">
         <is>
           <t>Monitor agy context</t>
         </is>
       </c>
-      <c r="C27" s="30" t="inlineStr">
+      <c r="C27" s="69" t="inlineStr">
         <is>
           <t>ag-context</t>
         </is>
       </c>
-      <c r="D27" s="14" t="n"/>
-    </row>
-    <row r="28" ht="409.6" customHeight="1" s="55">
-      <c r="A28" s="32" t="n">
+      <c r="D27" s="70" t="n"/>
+      <c r="E27" s="83" t="n"/>
+    </row>
+    <row r="28" ht="45" customHeight="1" s="55">
+      <c r="A28" s="67" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="33" t="inlineStr">
+      <c r="B28" s="68" t="inlineStr">
         <is>
           <t>🧠 Antigravity IDE: Strategic Fleet Advisor (المستشار التقني والاستراتيجي للأسطول)</t>
         </is>
       </c>
-      <c r="C28" s="34" t="inlineStr">
+      <c r="C28" s="69" t="inlineStr">
         <is>
           <t># Antigravity IDE: Strategic Fleet Advisor &amp; Technical Consultant Mode
 بصفتك الموجه والاستشاري الاستراتيجي الأول للمشروع (Chief Technical Advisor &amp; Fleet Consultant) في بيئة Antigravity IDE، تبدأ هذه الجلسة وتستمر وفقاً للبروتوكول المعماري التالي:
@@ -5441,22 +5720,23 @@
 أكد جاهزيتك فوراً لتقلد دور الموجه الاستراتيجي للأسطول لنبدأ العمل!</t>
         </is>
       </c>
-      <c r="D28" s="35" t="inlineStr">
+      <c r="D28" s="70" t="inlineStr">
         <is>
           <t>برومبت استراتيجي لتحويل Antigravity IDE إلى مستشار هندسي وموجه أول يحلل مخرجات وتقارير Claude Code بدقة، يشرح الـ Diffs وبوابات الجودة، ويولد أوامر التكليف بالإنجليزية للأسطول.</t>
         </is>
       </c>
+      <c r="E28" s="83" t="n"/>
     </row>
     <row r="29" ht="45" customHeight="1" s="55">
-      <c r="A29" s="36" t="n">
+      <c r="A29" s="67" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="37" t="inlineStr">
+      <c r="B29" s="68" t="inlineStr">
         <is>
           <t>📊 ag-context: Antigravity Context &amp; Token Monitor (أداة قياس ومراقبة استهلاك السياق والتوكنز)</t>
         </is>
       </c>
-      <c r="C29" s="38" t="inlineStr">
+      <c r="C29" s="69" t="inlineStr">
         <is>
           <t># فحص سريع لاستهلاك السياق الحالي ونسبة الامتلاء
 ag-context
@@ -5468,22 +5748,23 @@
 ag-context -j</t>
         </is>
       </c>
-      <c r="D29" s="39" t="inlineStr">
+      <c r="D29" s="70" t="inlineStr">
         <is>
           <t>أداة سريعة لقياس حجم سياق المحادثة (Context Tokens)، تفكير النموذج (Thinking)، والمخرجات بدقة 100% مباشرة من قاعدة بيانات جلسات Antigravity IDE، مع دعم المراقبة اللحظية والتاريخ وJSON.</t>
         </is>
       </c>
+      <c r="E29" s="83" t="n"/>
     </row>
     <row r="30" ht="45" customHeight="1" s="55">
-      <c r="A30" s="36" t="n">
+      <c r="A30" s="67" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="37" t="inlineStr">
+      <c r="B30" s="68" t="inlineStr">
         <is>
           <t>🧭 Antigravity Context Window Strategic Advisor (مستشار إدارة نافذة السياق وترشيد التوكنز)</t>
         </is>
       </c>
-      <c r="C30" s="38" t="inlineStr">
+      <c r="C30" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve"># استشارة استراتيجية سريعة حول حالة نافذة السياق والقرار الهندسي السليم
 context-advisor
@@ -5493,22 +5774,23 @@
 # "مستشار السياق" / "إدارة السياق" / "ترشيد السياق" / "قرارات السياق" </t>
         </is>
       </c>
-      <c r="D30" s="39" t="inlineStr">
+      <c r="D30" s="70" t="inlineStr">
         <is>
           <t>خطاف وأداة الاستشارة الاستراتيجية لتحليل استهلاك السياق في Antigravity IDE وتحديد منطقة الأمان (خضراء/صفراء/برتقالية/حمراء) واقتراح القرار الأمثل (استمرار/ترشيد/ضغط/تصفير استراتيجي).</t>
         </is>
       </c>
+      <c r="E30" s="83" t="n"/>
     </row>
     <row r="31" ht="45" customHeight="1" s="55">
-      <c r="A31" s="44" t="n">
+      <c r="A31" s="67" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="45" t="inlineStr">
+      <c r="B31" s="68" t="inlineStr">
         <is>
           <t>🏛️ الدستور المعماري الموحد والمدخل المزدوج للأسطول (Dual-Entry Fleet Architecture Protocol)</t>
         </is>
       </c>
-      <c r="C31" s="46" t="inlineStr">
+      <c r="C31" s="69" t="inlineStr">
         <is>
           <t>فعل بروتوكول المدخل المزدوج والدستور المعماري الموحد (AGENTS.md &amp; CLAUDE.md):
 1) اعتماد AGENTS.md كمرجع مركزي موحد لكافة بيئات الذكاء الاصطناعي (Codex, OpenCode, Cursor, Antigravity) واستيراده في CLAUDE.md لـ Claude Code.
@@ -5516,19 +5798,23 @@
 3) تفعيل جدول التوجيه الفوري (Instant Task Router) وتحديد مناطق الحجر الصحي للملفات الحساسة.</t>
         </is>
       </c>
-      <c r="D31" s="47" t="inlineStr">
+      <c r="D31" s="70" t="inlineStr">
         <is>
           <t>تأسيس المعمارية القياسية للمشاريع متعددة الوكلاء والـ CLIs عبر المدخل المزدوج الذكي، وضمان قراءة القواعد ذاتياً عبر كافة المنصات مع توجيه المهام وحماية الخصوصية طبقاً للقرار 19.</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="409.6" customHeight="1" s="55">
-      <c r="B33" s="29" t="inlineStr">
+      <c r="E31" s="83" t="n"/>
+    </row>
+    <row r="32" ht="45" customHeight="1" s="55">
+      <c r="A32" s="67" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="68" t="inlineStr">
         <is>
           <t>gheras</t>
         </is>
       </c>
-      <c r="C33" s="29" t="inlineStr">
+      <c r="C32" s="69" t="inlineStr">
         <is>
           <t>You are operating as the Master Orchestrator, Staff Architect, and Sole Testing Authority of the Autovemtech fleet (governed by CLAUDE.md, @AGENTS.md, @fleet_config.json, and @CURRENT_STATE.md).
 Mission: Execute Phase 1 Design &amp; Implementation for Clients/03_GHERAS_Center (EduTrack Pro), transforming the Luna 5.6 MVP (Clients/03_GHERAS_Center/تطبيق غراس.html) into a production-grade educational platform adhering strictly to the approved scope in @Clients/03_GHERAS_Center/06_Contracts_Invoices/GHERAS_GRAND_SLAM_OFFER.md.
@@ -5553,22 +5839,23 @@
 - Proceed autonomously through the milestones.</t>
         </is>
       </c>
-      <c r="D33" s="29" t="inlineStr">
+      <c r="D32" s="70" t="inlineStr">
         <is>
           <t>claude --dangerously-skip-permissions</t>
         </is>
       </c>
-    </row>
-    <row r="34" ht="65" customHeight="1" s="55">
-      <c r="A34" s="67" t="n">
-        <v>31</v>
-      </c>
-      <c r="B34" s="68" t="inlineStr">
+      <c r="E32" s="83" t="n"/>
+    </row>
+    <row r="33" ht="45" customHeight="1" s="55">
+      <c r="A33" s="67" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="68" t="inlineStr">
         <is>
           <t>🌱 تهيئة خريطة الكود وترشيد التوكنز عبر Graft (Init Codebase Context Map)</t>
         </is>
       </c>
-      <c r="C34" s="69" t="inlineStr">
+      <c r="C33" s="69" t="inlineStr">
         <is>
           <t># 1. تثبيت الأداة عالمياً عبر npm
 npm install -g @nanonets/graft
@@ -5576,36 +5863,71 @@
 graft init --agents claude</t>
         </is>
       </c>
-      <c r="D34" s="70" t="inlineStr">
+      <c r="D33" s="70" t="inlineStr">
         <is>
           <t>بناء خريطة سياقية معرفية مستدامة للأكواد في مجلد graft/ لترشيد استهلاك كوتا Claude Code والأسطول بنسبة 42% وتقليل استدعاءات الأدوات بنسبة 46% وتسريع الاستجابة 60% عبر التحليل الشجري الثابت ($0 tree-sitter AST).</t>
         </is>
       </c>
-    </row>
-    <row r="35" ht="50" customHeight="1" s="55">
-      <c r="A35" s="67" t="n">
-        <v>32</v>
-      </c>
-      <c r="B35" s="68" t="inlineStr">
+      <c r="E33" s="83" t="n"/>
+    </row>
+    <row r="34" ht="45" customHeight="1" s="55">
+      <c r="A34" s="67" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="68" t="inlineStr">
         <is>
           <t>⚡ تشغيل وتهيئة Graft المباشرة عبر npx (Graft One-Shot Run)</t>
         </is>
       </c>
-      <c r="C35" s="69" t="inlineStr">
+      <c r="C34" s="69" t="inlineStr">
         <is>
           <t># تشغيلها مباشرة دون تثبيت عام عبر npx:
 npx @nanonets/graft init</t>
         </is>
       </c>
+      <c r="D34" s="70" t="inlineStr">
+        <is>
+          <t>تشغيل وتهيئة خريطة الكود وبناء مجلد graft/ وربط خطافات Claude Code مباشرة بنقرة واحدة دون الحاجة لتثبيت الحزمة عالمياً على النظام.</t>
+        </is>
+      </c>
+      <c r="E34" s="83" t="n"/>
+    </row>
+    <row r="35" ht="45" customHeight="1" s="55">
+      <c r="A35" s="67" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="68" t="inlineStr">
+        <is>
+          <t>⚡ قيادة الأسطول: إطلاق عاملي GLM 5.3 Flash بالتوازي وتطهير الواجهات (Dual-GLM Parallel Fleet)</t>
+        </is>
+      </c>
+      <c r="C35" s="69" t="inlineStr">
+        <is>
+          <t>Role: Master Orchestrator (Claude Code CLI / Opus Max)
+Mission: Coordinate parallel fleet execution with dual GLM 5.3 Flash workers and enforce executive UI purification.
+Directives:
+1. Parallel Dual-GLM Execution:
+   - Launch TWO parallel GLM 5.3 Flash workers concurrently across non-colliding tasks:
+     * Worker A (OpenCode CLI): opencode run --auto -m opencode-go/glm-5.3-flash for terminal commands, data layers, or backend tasks.
+     * Worker B (Cline CLI / Secondary OpenCode): cline or parallel instance on distinct files for UI scaffolding, component refactoring, or validation.
+   - Ensure zero race conditions by assigning completely disjoint file sets to each worker.
+2. Executive UI Sanitization Standard:
+   - Purge all internal development tags, requirement IDs (Req 1-5, 'المتطلب'), and debug comments from client-facing web applications.
+   - Convert all titles and labels to professional, business-grade Arabic terminology suitable for executive presentation.
+3. Exclusive Quality &amp; Verification Gate:
+   - Sole authority for testing, lint verification, and [APPROVED] architectural sign-offs remains with Claude Code CLI.</t>
+        </is>
+      </c>
       <c r="D35" s="70" t="inlineStr">
         <is>
-          <t>تشغيل وتهيئة خريطة الكود وبناء مجلد graft/ وربط خطافات Claude Code مباشرة بنقرة واحدة دون الحاجة لتثبيت الحزمة عالمياً على النظام.</t>
-        </is>
-      </c>
+          <t>أمر قيادة الأسطول الموجه لـ Claude Code CLI لإطلاق عاملي GLM 5.3 Flash بالتوازي لمهام متزامنة وتطبيق معيار التطهير التنفيذي للواجهات.</t>
+        </is>
+      </c>
+      <c r="E35" s="83" t="n"/>
     </row>
     <row r="36" ht="45" customHeight="1" s="55">
       <c r="A36" s="67" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B36" s="68" t="inlineStr">
         <is>
@@ -5625,29 +5947,7 @@
           <t>توجيه قيادي صارم يلزم Claude Code CLI (Opus Max) بتفكيك المهام البرمجية وتشغيل 2 إلى 4 عمال من نموذج GLM 5.3 Flash بالتوازي عبر OpenCode CLI و Cline CLI على مسارات ملفات غير متصادمة، مما يعظم سرعة الإنجاز بنسبة 300%+ ويحفظ ميزانية توكنز كلود للمراجعات المعمارية واحتكار الاختبارات حصرياً.</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="45" customHeight="1" s="55">
-      <c r="A37" s="67" t="n">
-        <v>34</v>
-      </c>
-      <c r="B37" s="68" t="inlineStr">
-        <is>
-          <t>⚡ التوجيه الإلزامي لـ Claude لتشغيل عمال GLM 5.3 Flash بالتوازي (Multi-Worker Parallel Dispatch)</t>
-        </is>
-      </c>
-      <c r="C37" s="69" t="inlineStr">
-        <is>
-          <t>Act as Master Orchestrator (Claude Opus Max). You are commanded to actively dispatch two or more GLM 5.3 Flash workers in parallel across non-colliding scopes:
-1. Worker A (OpenCode CLI): &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_A_prompt}"
-2. Worker B (Cline CLI / Parallel OpenCode): &amp; cline "{task_B_prompt}" OR &amp; opencode run -m opencode-go/glm-5.3-flash --auto "{task_B_prompt}"
-Decompose independent sub-tasks, launch workers simultaneously in background, enforce disjoint file paths, and retain exclusive authority for architecture reviews and test approvals [APPROVED].</t>
-        </is>
-      </c>
-      <c r="D37" s="70" t="inlineStr">
-        <is>
-          <t>توجيه قيادي صارم يلزم Claude Code CLI (Opus Max) بتفكيك المهام البرمجية وتشغيل 2 إلى 4 عمال من نموذج GLM 5.3 Flash بالتوازي عبر OpenCode CLI و Cline CLI على مسارات ملفات غير متصادمة، مما يعظم سرعة الإنجاز بنسبة 300%+ ويحفظ ميزانية توكنز كلود للمراجعات المعمارية واحتكار الاختبارات حصرياً.</t>
-        </is>
-      </c>
+      <c r="E36" s="83" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5661,7 +5961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -5692,216 +5992,226 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="31.95" customHeight="1" s="55">
-      <c r="A2" s="11" t="n">
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="68" t="inlineStr">
         <is>
           <t>العصف الذهني والتصميم التفاعلي</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:brainstorming)</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="70" t="inlineStr">
         <is>
           <t>استبيان تفاعلي لاستكشاف متطلبات المستخدم وتصميم المعمارية قبل البدء في كتابة الأكواد.</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.95" customHeight="1" s="55">
-      <c r="A3" s="11" t="n">
+      <c r="E2" s="83" t="n"/>
+    </row>
+    <row r="3" ht="45" customHeight="1" s="55">
+      <c r="A3" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>كتابة خطط التنفيذ البرمجية</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:writing-plans)</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="70" t="inlineStr">
         <is>
           <t>صياغة خطة عمل تفصيلية تتضمن متطلبات المراجعة، التعديلات المقترحة، وخطة التحقق والاختبار.</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="31.95" customHeight="1" s="55">
-      <c r="A4" s="11" t="n">
+      <c r="E3" s="83" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="55">
+      <c r="A4" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>التطوير الموجه بالاختبارات (TDD)</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:test-driven-development)</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>كتابة اختبارات الوحدة الفاشلة أولاً ثم كتابة كود الإنتاج الأدنى الكافي لاجتيازها بنجاح.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="31.95" customHeight="1" s="55">
-      <c r="A5" s="11" t="n">
+      <c r="E4" s="83" t="n"/>
+    </row>
+    <row r="5" ht="45" customHeight="1" s="55">
+      <c r="A5" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>التحقق الصارم قبل التسليم</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:verification-before-completion)</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>إلزام النموذج بتشغيل أوامر الفحص والـ Tests والتأكد من مخرجاتها قبل إعلان اكتمال المهمة.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="31.95" customHeight="1" s="55">
-      <c r="A6" s="11" t="n">
+      <c r="E5" s="83" t="n"/>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="55">
+      <c r="A6" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>التطوير عبر الوكلاء الفرعيين (SDD)</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:subagent-driven-development)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>تقسيم الخطة إلى مهام مستقلة وتوزيعها على وكلاء فرعيين متوازيين مع نقاط مراجعة.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="31.95" customHeight="1" s="55">
-      <c r="A7" s="11" t="n">
+      <c r="E6" s="83" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="55">
+      <c r="A7" s="67" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>منهجية تصحيح الأعطال المنهجية</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:systematic-debugging)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>معالجة الأعطال بـ 5 خطوات: إعادة الإنتاج -&gt; العزل -&gt; التحليل -&gt; الفرضية -&gt; التثبيت والتأكيد.</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="31.95" customHeight="1" s="55">
-      <c r="A8" s="11" t="n">
+      <c r="E7" s="83" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1" s="55">
+      <c r="A8" s="67" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>عزل العمل عبر Git Worktrees</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:using-git-worktrees)</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>إنشاء مساحة عمل معزولة للميزات الجديدة لتفادي تلويث الفرع الرئيسي أثناء التطوير.</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="31.95" customHeight="1" s="55">
-      <c r="A9" s="11" t="n">
+      <c r="E8" s="83" t="n"/>
+    </row>
+    <row r="9" ht="45" customHeight="1" s="55">
+      <c r="A9" s="67" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="68" t="inlineStr">
         <is>
           <t>استقبال ومراجعة الكود</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:receiving-code-review)</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>التعامل مع ملاحظات المراجعين البرمجيين والتحقق الفني الصارم قبل تطبيق التعديلات.</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="31.95" customHeight="1" s="55">
-      <c r="A10" s="11" t="n">
+      <c r="E9" s="83" t="n"/>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="55">
+      <c r="A10" s="67" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>طلب مراجعة الكود قبل الدمج</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:requesting-code-review)</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>توليد طلب فحص الجودة والأمان والتأكد من مطابقة الكود للمعايير قبل عمل الـ PR.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="31.95" customHeight="1" s="55">
-      <c r="A11" s="11" t="n">
+      <c r="E10" s="83" t="n"/>
+    </row>
+    <row r="11" ht="45" customHeight="1" s="55">
+      <c r="A11" s="67" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="68" t="inlineStr">
         <is>
           <t>إنهاء ودمج فرع التطوير</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:finishing-a-development-branch)</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="70" t="inlineStr">
         <is>
           <t>الخطوات الآمنة لدمج الفرع، تشغيل الاختبارات النهائية، وتنظيف بيئات العمل المؤقتة.</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="48" customHeight="1" s="55">
-      <c r="A12" s="15" t="n">
+      <c r="E11" s="83" t="n"/>
+    </row>
+    <row r="12" ht="45" customHeight="1" s="55">
+      <c r="A12" s="67" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="68" t="inlineStr">
         <is>
           <t>قالب تفويض كلود كمهندس وموجه (Orchestrator)</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="69" t="inlineStr">
         <is>
           <t>[ROLE &amp; ARCHITECTURE: YOU ARE THE LEAD ORCHESTRATOR &amp; QA AUDITOR]
 You are the Chief Software Architect and QA Gatekeeper adhering to amElnagdy/delegate-skills architecture. Antigravity IDE is your Fast Implementer.
@@ -5913,42 +6223,44 @@
    - IF VERIFIED &amp; GREEN: Issue [APPROVED], create the Git commit, and proceed to the next brief.</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>قالب تكليف كلود كمهندس معماري ومدقق جودة، يقوم بإصدار المهام وتدقيق واختبار الكود بنفسه وإصدار توجيهات التصحيح حتى اجتياز الفحص 100%.</t>
         </is>
       </c>
+      <c r="E12" s="83" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1" s="55">
-      <c r="A13" s="44" t="n">
+      <c r="A13" s="67" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="45" t="inlineStr">
+      <c r="B13" s="68" t="inlineStr">
         <is>
           <t>🎨 نظام واجهات ThreeUI ثلاثية الأبعاد (ThreeUI 3D Web Components)</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="69" t="inlineStr">
         <is>
           <t>استدعِ مهارة [threeui-design-system] لبناء واجهة ويب ثلاثية الأبعاد تفاعلية: 1) إنشاء مشهد Three.js بطل (Hero Canvas) أو بطاقات Spatial Glassmorphism مع تفاعل مؤشر الفأرة (Mouse Orbit). 2) تطبيق تدرجات الشيدر المتوهجة وخلفيات الجسيمات بنمط النيون الداكن. 3) فرض معيار التنظيف الصارم للذاكرة (dispose geometries/materials/renderer) لمنع تسريب WebGL وتحقيق 60 FPS مع بديل متجاوب للهواتف.</t>
         </is>
       </c>
-      <c r="D13" s="47" t="inlineStr">
+      <c r="D13" s="70" t="inlineStr">
         <is>
           <t>بناء واجهات ومكونات ويب ثلاثية الأبعاد غامرة وعالية الأداء بالاعتماد على معمارية Meng To ومكتبة ThreeUI مع الحفاظ الكامل على سهولة الوصول ومنع تسريب الذاكرة.</t>
         </is>
       </c>
+      <c r="E13" s="83" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1" s="55">
-      <c r="A14" s="44" t="n">
+      <c r="A14" s="67" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="45" t="inlineStr">
+      <c r="B14" s="68" t="inlineStr">
         <is>
           <t>قيادة السبرنت الذاتي للأسطول عبر Claude Code Master Orchestrator 👑</t>
         </is>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="69" t="inlineStr">
         <is>
           <t>You are operating as the Master Orchestrator, Staff Architect, and Sole Testing Authority of the Autovemtech fleet (governed by CLAUDE.md, @AGENTS.md, @fleet_config.json, and @CURRENT_STATE.md).
 Mission: Execute an uninterrupted 8-hour autonomous development sprint for Clients/03_GHERAS_Center (EduTrack Pro), transforming the Luna 5.6 MVP (Clients/03_GHERAS_Center/تطبيق غراس.html) into a production-grade educational platform.
@@ -5969,11 +6281,12 @@
 - Update @CURRENT_STATE.md after each completed milestone so Antigravity IDE can debrief the developer in Arabic.</t>
         </is>
       </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="D14" s="70" t="inlineStr">
         <is>
           <t>الموجه القيادي لـ Claude Code CLI كـ Master Orchestrator لتشغيل سبرنت ذاتي (8 ساعات) دون انقطاع، مع تفويض المهام الروتينية لـ OpenCode و Codex، واحتكار الفحص والاعتماد لـ Claude، وتحديث CURRENT_STATE.md ليتمكن المطور من متابعة المنجزات عبر Antigravity IDE باللغة العربية.</t>
         </is>
       </c>
+      <c r="E14" s="83" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1" s="55">
       <c r="A15" s="67" t="n">
@@ -6011,6 +6324,7 @@
           <t>موجه هندسي مؤتمت لتنفيذ رفع ونشر تحديثات واجهة الويب لمنصة EduTrack Pro على سيرفر Hostinger VPS (187.55.226.225) لمركز غراس عبر Caddy و Docker، مع إجراء اختبارات الدخان (Smoke Test) والتحقق الحي من صلاحيات المشرفين وروابط المعاينة.</t>
         </is>
       </c>
+      <c r="E15" s="83" t="n"/>
     </row>
     <row r="16" ht="45" customHeight="1" s="55">
       <c r="A16" s="67" t="n">
@@ -6031,6 +6345,7 @@
           <t>محرك المراجعة التنافسية (debate-review): تشغيل نموذجين مختلفين لتمزيق النقاط العمياء ومناظرة كل ملاحظة قبل اعتمادها كتعليق سطري متفق عليه أو متنازع عليه.</t>
         </is>
       </c>
+      <c r="E16" s="83" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1" s="55">
       <c r="A17" s="67" t="n">
@@ -6051,6 +6366,7 @@
           <t>وكيل المتابعة المستمرة (babysit-pr): حصاد كافة ملاحظات المراجعين على الـ PR، التحقق منها على الكود الحي، إصلاح المشاكل الحقيقية، والرد في الخيوط وإعادة الفحص حتى الدمج.</t>
         </is>
       </c>
+      <c r="E17" s="83" t="n"/>
     </row>
     <row r="18" ht="45" customHeight="1" s="55">
       <c r="A18" s="67" t="n">
@@ -6058,19 +6374,41 @@
       </c>
       <c r="B18" s="68" t="inlineStr">
         <is>
+          <t>🚀 توجيه الأسطول لتطوير وإصلاح ميزات الويب (Fleet Feature Dispatch &amp; Fix)</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>بسم الله. ابدأ الميزة. وجه الاسطول قم بإصلاح زر التنزيل في تطبيق الويب eduTrack Pro الخاص بالعميل مركز غراس</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="inlineStr">
+        <is>
+          <t>أمر إطلاق وتوجيه أسطول الـ CLIs لبدء دورة هندسة وتدقيق الميزات في EduTrack Pro وفق بروتوكول الخطوة صفر وبوابة تدقيق Claude Code الحصرية.</t>
+        </is>
+      </c>
+      <c r="E18" s="83" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1" s="55">
+      <c r="A19" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="68" t="inlineStr">
+        <is>
           <t>🌊 توجيه الموجة المعمارية المستقلة والتوزيع المتوازي للأسطول (Google Stitch &amp; Operations Control)</t>
         </is>
       </c>
-      <c r="C18" s="69" t="inlineStr">
+      <c r="C19" s="69" t="inlineStr">
         <is>
           <t># 🌊 AUTONOMOUS WAVE EXECUTION &amp; MULTI-AGENT PARALLEL DIRECTIVE\n\nTarget: Claude Code CLI (Opus Max — Master Orchestrator &amp; Sole Testing Monopoly)\nParallel Workers: OpenCode CLI (GLM 5.3 Flash), Cline CLI, Antigravity CLI (agcli)\nDesign Paradigm: Google Stitch &amp; Dribbble Operations Control (Micro-Sparklines, Icon Navigation Rail, Outcomes Matrix)\nWorkspace: f:\AI PROJECTS\Claude+Antigravity -production\taj_al_waqar_global\n\nExecution Protocol:\n1. Analyze: Inspect newly authored code under lib/ for clean static analysis.\n2. Author Tests: Comprehensive unit and widget tests under test/ for all domain contracts &amp; widgets.\n3. Execute Verification Suite: C:\flutter_sdk\bin\flutter test --concurrency=1 (0 failures, 0 regressions).\n4. Certification: Inscribe formal ADR in MEMORY_STORE.md and grant [APPROVED TO SHIP] in FLEET_LOG.md.</t>
         </is>
       </c>
-      <c r="D18" s="70" t="inlineStr">
+      <c r="D19" s="70" t="inlineStr">
         <is>
           <t>موجه قيادي معتمد لتنفيذ موجات التطوير البرمجي بالأسطول المتوازي، مع الالتزام الصارم بمعايير Google Stitch ولوحات تحكم Dribbble ومونوپولي الاختبارات لكلود كود.</t>
         </is>
       </c>
+      <c r="E19" s="83" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6083,7 +6421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6114,216 +6452,226 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="31.95" customHeight="1" s="55">
-      <c r="A2" s="11" t="n">
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="68" t="inlineStr">
         <is>
           <t>حارس إثبات الحقائق</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>Gate: [Fact-Forcing Gate]</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="70" t="inlineStr">
         <is>
           <t>يمنع إنشاء أو تعديل أي ملف كودي إلا بعد فحص شجرة المشروع وإثبات عدم التكرار وصحة المسار.</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.95" customHeight="1" s="55">
-      <c r="A3" s="11" t="n">
+      <c r="E2" s="83" t="n"/>
+    </row>
+    <row r="3" ht="45" customHeight="1" s="55">
+      <c r="A3" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>حارس منع الإنهاء دون تحقق</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="69" t="inlineStr">
         <is>
           <t>Gate: [Block-No-Verify Gate]</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="70" t="inlineStr">
         <is>
           <t>يمنع إنهاء التذكرة أو ادعاء النجاح إذا لم يقم النموذج بتشغيل الاختبارات وإثبات صحة النتيجة.</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="31.95" customHeight="1" s="55">
-      <c r="A4" s="11" t="n">
+      <c r="E3" s="83" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="55">
+      <c r="A4" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>خطاف بدء الجلسة</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>Hook: session-start.js</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>تهيئة المتغيرات، حقن القواعد البرمجية الصارمة، وضبط مسارات الأدوات عند فتح أي جلسة.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="31.95" customHeight="1" s="55">
-      <c r="A5" s="11" t="n">
+      <c r="E4" s="83" t="n"/>
+    </row>
+    <row r="5" ht="45" customHeight="1" s="55">
+      <c r="A5" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>خطاف ما قبل الضغط</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="69" t="inlineStr">
         <is>
           <t>Hook: pre-compact.js</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>استخراج وتلخيص الدروس المستفادة والقرارات المعمارية وحفظها في الذاكرة قبل ضغط السياق.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="31.95" customHeight="1" s="55">
-      <c r="A6" s="11" t="n">
+      <c r="E5" s="83" t="n"/>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="55">
+      <c r="A6" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>خطاف حراسة الأوامر الطرفية</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="69" t="inlineStr">
         <is>
           <t>Hook: before-shell-execution.js</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>فحص الأوامر الطرفية واعتراض الأوامر الخطيرة لمنع حذف الملفات أو تسريب البيانات.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="31.95" customHeight="1" s="55">
-      <c r="A7" s="11" t="n">
+      <c r="E6" s="83" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="55">
+      <c r="A7" s="67" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>خطاف ما بعد تعديل الملفات</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="69" t="inlineStr">
         <is>
           <t>Hook: after-file-edit.js</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>تشغيل الفاحص اللغوي (Linter) أو منسق الأكواد آلياً فور تعديل أي ملف لضمان الاتساق.</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="31.95" customHeight="1" s="55">
-      <c r="A8" s="11" t="n">
+      <c r="E7" s="83" t="n"/>
+    </row>
+    <row r="8" ht="45" customHeight="1" s="55">
+      <c r="A8" s="67" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>خطاف بدء الوكلاء الفرعيين</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>Hook: subagent-start.js</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>تزويد الوكيل الفرعي بسياق المهمة المعزول وقواعد المشروع قبل بدء التنفيذ.</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="31.95" customHeight="1" s="55">
-      <c r="A9" s="11" t="n">
+      <c r="E8" s="83" t="n"/>
+    </row>
+    <row r="9" ht="45" customHeight="1" s="55">
+      <c r="A9" s="67" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="68" t="inlineStr">
         <is>
           <t>خطاف إيقاف الجلسة والإنهاء</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="69" t="inlineStr">
         <is>
           <t>Hook: session-end.js</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="70" t="inlineStr">
         <is>
           <t>أخذ لقطة لملف الـ Diff وتوثيق المنجزات تلقائياً في MEMORY_STORE.md قبل إغلاق الجلسة.</t>
         </is>
       </c>
+      <c r="E9" s="83" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1" s="55">
-      <c r="A10" s="40" t="n">
+      <c r="A10" s="67" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="41" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>🧹 خطاف ترحيل وتطهير أدوات المحرر (Hook 28: Workspace Sanitizer)</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="69" t="inlineStr">
         <is>
           <t>evacuate-tools --project "."</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>فحص ومزامنة أدوات المحرر مع Global Config، وترحيل كافة الأدلة والمستندات والسكربتات إلى المستودع المركزي Claude+Antigravity بعد التحقق التشفيري SHA-256، وتنظيف مخلفات JVM لاستعادة نقاء سياق المشروع 100%.</t>
         </is>
       </c>
+      <c r="E10" s="83" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1" s="55">
-      <c r="A11" s="44" t="n">
+      <c r="A11" s="67" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="45" t="inlineStr">
+      <c r="B11" s="68" t="inlineStr">
         <is>
           <t>🛡️ درع الفحص الأمني السداسي لكود الـ AI (Vibe Coding Security Shield)</t>
         </is>
       </c>
-      <c r="C11" s="46" t="inlineStr">
+      <c r="C11" s="69" t="inlineStr">
         <is>
           <t>فعل خطاف الفحص الأمني ودرع Vibe Coding (خطاف 8) لفحص المشروع بالكامل عبر الركائز الست: 1) فحص كود المصدر عبر Semgrep لكشف ثغرات الحقن والمنطق. 2) مسح الأسرار والمفاتيح عبر Gitleaks ومنع تسريبها للـ Git history. 3) فحص التبعيات وصور Docker عبر Trivy لكشف ثغرات CVEs وتوليد الـ SBOM. 4) الفحص الديناميكي DAST عبر OWASP ZAP ضد نقاط الـ API والـ Web app. 5) فحص أخطاء البنية التحتية والـ Dockerfile عبر Checkov. 6) ضبط ملف renovate.json لأتمتة تحديث التبعيات عبر PRs.</t>
         </is>
       </c>
-      <c r="D11" s="47" t="inlineStr">
+      <c r="D11" s="70" t="inlineStr">
         <is>
           <t>تفعيل منظومة الحماية المتكاملة لمطوري الـ AI والـ Vibe Coding لتأمين الأكواد والمفاتيح والتبعيات والحاويات والبنية التحتية قبل الرفع لبيئة الإنتاج.</t>
         </is>
       </c>
+      <c r="E11" s="83" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1" s="55">
-      <c r="A12" s="44" t="n">
+      <c r="A12" s="67" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="45" t="inlineStr">
+      <c r="B12" s="68" t="inlineStr">
         <is>
           <t>🧹 تنظيم وهيكلة مسار مساحة العمل وتطهير الجذر (Workspace Path &amp; Root Sanitation)</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="69" t="inlineStr">
         <is>
           <t>رتب المسار, نظم المجلد, ترتيب مسار
 # التوجيه الهندسي الشامل:
@@ -6333,17 +6681,16 @@
 3) أرشفة الشهادات التدريبية في مجلدات فرعية، وحذف ملفات القفل المؤقتة والمجلدات الفارغة.</t>
         </is>
       </c>
-      <c r="D12" s="47" t="inlineStr">
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>أمر نوعي لإعادة هيكلة وتطهير مسار مساحة العمل، فرز ملفات الـ PDF، تصحيح مسارات العملاء، وعزل وثائق الحسابات الرسمية والشهادات وفق المعيار 18 لمنع تلوث جذر المشروع.</t>
         </is>
       </c>
+      <c r="E12" s="83" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1" s="55">
-      <c r="A13" s="67" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
+      <c r="A13" s="67" t="n">
+        <v>12</v>
       </c>
       <c r="B13" s="68" t="inlineStr">
         <is>
@@ -6361,6 +6708,7 @@
           <t>تشغيل مستمع تليجرام في الخلفية كـ Task مستقل لمراقبة الرسائل والأوامر الصوتية من الجوال، وحفظ الطلبات في telegram_request.json، وتحويل البصمات الصوتية OGG إلى WAV عبر PyAV، وإيقاظ Antigravity IDE تلقائياً بإشارة الأولوية القصوى لمعالجة الطلب والرد على الهاتف عبر send_reply.py.</t>
         </is>
       </c>
+      <c r="E13" s="83" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1" s="55">
       <c r="A14" s="67" t="n">
@@ -6381,6 +6729,7 @@
           <t>بوابة حراسة كود ووردبريس (wp-guard): فحص التعقيم والهروب، الـ Nonces، وصلاحيات المستخدم، وحماية استعلامات $wpdb-&gt;prepare، ودعم اللغات المتعددة i18n والأداء.</t>
         </is>
       </c>
+      <c r="E14" s="83" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1" s="55">
       <c r="A15" s="67" t="n">
@@ -6401,6 +6750,7 @@
           <t>بوابة حراسة ووكومرس (woo-guard): حراسة العمليات المالية، منع الالتفاف على كائنات HPOS CRUD، تأمين الـ Checkout ومطابقة معايير الدفع وتجنب استخدام الـ Floats للأموال.</t>
         </is>
       </c>
+      <c r="E15" s="83" t="n"/>
     </row>
     <row r="16" ht="45" customHeight="1" s="55">
       <c r="A16" s="67" t="n">
@@ -6421,6 +6771,7 @@
           <t>أمر تشغيلي ملزم لكافة وكلاء الأسطول يفرض إنجاز المهام بأصغر تغيير كافٍ مع معالجة الخلل من الجذر ومنع الترقيع السطحي، وتنسيق الفحص مع احتكار Claude للاختبارات وترشيد استهلاك السياق.</t>
         </is>
       </c>
+      <c r="E16" s="83" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1" s="55">
       <c r="A17" s="67" t="n">
@@ -6441,6 +6792,49 @@
           <t>تفعيل الخطاف رقم 29 لمعايرة وترقية مصفوفة نماذج أسطول الـ CLIs لاعتماد Claude 5.5 Opus Max و Claude Sonnet 5.5 وتحديث قيود [C-11] و [C-21] و [C-38] وملفات fleet_config.json وسجلات الذاكرة.</t>
         </is>
       </c>
+      <c r="E17" s="83" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="55">
+      <c r="A18" s="67" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="68" t="inlineStr">
+        <is>
+          <t>📚 حزمة مهارات ومبادئ pstack للأسطول (pstack Fleet Engineering Suite &amp; Principles)</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>Skill(pstack:unslop); Skill(pstack:blast-radius); Skill(pstack:arena); Skill(pstack:correct); Skill(pstack:create-verification-skill) / "استدعِ مهارات pstack" / "pstack suite"</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="inlineStr">
+        <is>
+          <t>حزمة المهارات والمبادئ الهندسية الـ 12 المعتمدة من مستودع backnotprop/pstack للمهندسة Lauren Tan (فريق React Core ومطورة Meta/Netflix/Cursor السابقة) المعتمدة لأسطول Autovemtech لمكافحة الكود الهش وحشو الذكاء الاصطناعي (Anti-Slop AI Code)، وانضباط الحدود، ونظام الأنواع، وتطعيم الحلول المعمارية، وتثبيت الأخطاء في CI.</t>
+        </is>
+      </c>
+      <c r="E18" s="83" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1" s="55">
+      <c r="A19" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="68" t="inlineStr">
+        <is>
+          <t>📖 دليل الاستخدام الشامل لمهارات pstack المعتمدة للأسطول (pstack Fleet Engineering Guide)</t>
+        </is>
+      </c>
+      <c r="C19" s="69" t="inlineStr">
+        <is>
+          <t>view_file docs/PSTACK_FLEET_GUIDE.md / "دليل مهارات pstack" / "pstack fleet guide" / "عرض دليل pstack"</t>
+        </is>
+      </c>
+      <c r="D19" s="70" t="inlineStr">
+        <is>
+          <t>الدليل الشامل لاستخدام واستدعاء مهارات ومبادئ pstack الـ 12 المعتمدة في أسطول Autovemtech لمكافحة حشو الكود (Anti-slop) وانضباط الحدود وتثبيت الاختبارات وتنافس النماذج، ومسارات العمل المعتمدة للأسطول.</t>
+        </is>
+      </c>
+      <c r="E19" s="83" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6453,7 +6847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6484,145 +6878,152 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="31.95" customHeight="1" s="55">
-      <c r="A2" s="11" t="n">
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="68" t="inlineStr">
         <is>
           <t>البحث المعمق والاستكشاف</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:deep-research)</t>
         </is>
       </c>
-      <c r="D2" s="14" t="inlineStr">
+      <c r="D2" s="70" t="inlineStr">
         <is>
           <t>البحث العميق في وثائق المكتبات، الأبحاث، والأكواد المصدرية لاستخراج الحلول المثلى.</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.95" customHeight="1" s="55">
-      <c r="A3" s="11" t="n">
+      <c r="E2" s="83" t="n"/>
+    </row>
+    <row r="3" ht="45" customHeight="1" s="55">
+      <c r="A3" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="68" t="inlineStr">
         <is>
           <t>حلقة التحقق المغلقة الذاتية</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:verification-loop)</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="70" t="inlineStr">
         <is>
           <t>حلقة فحص ذاتية مغلقة تقوم باكتشاف أخطاء الترجمة والبناء وإصلاحها تلقائياً.</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="31.95" customHeight="1" s="55">
-      <c r="A4" s="11" t="n">
+      <c r="E3" s="83" t="n"/>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="55">
+      <c r="A4" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>بناء وتطوير المهارات</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:writing-skills)</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>إنشاء مهارات تخصصية جديدة مع وثائق SKILL.md وترويسة YAML قياسية وأمثلة تطبيقية.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="31.95" customHeight="1" s="55">
-      <c r="A5" s="11" t="n">
+      <c r="E4" s="83" t="n"/>
+    </row>
+    <row r="5" ht="45" customHeight="1" s="55">
+      <c r="A5" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="68" t="inlineStr">
         <is>
           <t>الذاكرة المستدامة الموحدة</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C5" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:unified-memory)</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="70" t="inlineStr">
         <is>
           <t>إدارة الذاكرة اللامركزية وحفظ الدروس والقرارات وتصدير السياق للوكلاء.</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="31.95" customHeight="1" s="55">
-      <c r="A6" s="11" t="n">
+      <c r="E5" s="83" t="n"/>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="55">
+      <c r="A6" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>تحسين الأداء وإدارة الموارد</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:performance-optimizer)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="70" t="inlineStr">
         <is>
           <t>فحص اختناقات الأداء، منع عمليات إعادة الرسم في Compose، وضبط استهلاك الذاكرة.</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="31.95" customHeight="1" s="55">
-      <c r="A7" s="11" t="n">
+      <c r="E6" s="83" t="n"/>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="55">
+      <c r="A7" s="67" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>التوزيع المتوازي للوكلاء</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="69" t="inlineStr">
         <is>
           <t>Skill(superpowers:dispatching-parallel-agents)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>توزيع المهام الكبيرة على وكلاء فرعيين مستقلين وتجميع المخرجات بكفاءة وسرعة.</t>
         </is>
       </c>
+      <c r="E7" s="83" t="n"/>
     </row>
     <row r="8" ht="45" customHeight="1" s="55">
-      <c r="A8" s="44" t="n">
+      <c r="A8" s="67" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="45" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>🚀 مستشار هورموزي لنمو البيزنس وصناعة العروض (Hormozi Business &amp; Offer Advisor)</t>
         </is>
       </c>
-      <c r="C8" s="46" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>استدعِ وكيل مستشار هورموزي [hormozi-growth-advisor] لتحليل نموذج العمل الحالي وتطبيق أطر $100M: 1) صياغة Grand Slam Offer يطبق معادلة القيمة (تعظيم النتيجة المأمولة والاحتمالية وتقليص الوقت والجهد للصفر). 2) تحديد مرحلة المشروع الحالية ضمن مصفوفة التوسع الـ 10 مراحل (من Improvise إلى Capitalize) وحصر التركيز في أولويتها التكتيكية. 3) تطبيق دليل التسعير بالقيمة (Value-Based Pricing) أو خطة رفع الأسعار دون فقدان العملاء.</t>
         </is>
       </c>
-      <c r="D8" s="47" t="inlineStr">
+      <c r="D8" s="70" t="inlineStr">
         <is>
           <t>استشارة استراتيجية وتكتيكية لنمو المشاريع الرقمية والبرمجية، هندسة العروض التي لا تُقاوم، وتحديد مرحلة التوسع ومضاعفة القيمة والإيرادات وفق منهجية أليكس هورموزي.</t>
         </is>
       </c>
+      <c r="E8" s="83" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1" s="55">
       <c r="A9" s="67" t="n">
@@ -6657,6 +7058,7 @@
           <t>هندسة وتوليد برومبتات سينمائية فائقة الواقعية (8K Photorealism) للصور والفيديوهات الإعلانية لعملاء الوكالة استناداً لمعايير MeiGen.ai ومحركات FLUX و Midjourney و Runway، مع تحديد الكاميرا والإضاءة والعدسات بدقة احترافية.</t>
         </is>
       </c>
+      <c r="E9" s="83" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1" s="55">
       <c r="A10" s="67" t="n">
@@ -6664,19 +7066,20 @@
       </c>
       <c r="B10" s="68" t="inlineStr">
         <is>
-          <t>🎨 تصميم وبناء مواصفات DESIGN.md (Design MD Architect)</t>
+          <t>🧪 منظومة الاختبارات الوكيلية الشاملة e2e ومولد مهارات التحقق</t>
         </is>
       </c>
       <c r="C10" s="69" t="inlineStr">
         <is>
-          <t>design-md-architect: أنشئ ملف DESIGN.md متكامل للمشروع وفق مواصفات Google Stitch و Refero Styles مع ضبط باليت الألوان الدلالية، ومقاييس الخطوط والتباعد، وقواعد RTL.</t>
+          <t>e2e init; e2e run; /create-verification-skill</t>
         </is>
       </c>
       <c r="D10" s="70" t="inlineStr">
         <is>
-          <t>توليد وتوحيد مواصفات DESIGN.md المرجعية للمشروع لضمان التماسك البصري لكافة وكلاء الذكاء الاصطناعي (Claude Code, Cursor, Codex, Gemini, Antigravity) ومنع العشوائية.</t>
-        </is>
-      </c>
+          <t>إطار عمل ثوري مفتوح المصدر (tester-army/e2e) لقيادة اختبارات الويب والموبايل (@e2e-dev/web, @e2e-dev/mobile) بأهداف وكيلية طبيعية (agent.act, agent.assert) وتأكيدات قطعية، مع تقنية الـ Replay Cache الحصرية (إعادة تشغيل الاختبارات المؤكدة بـ 0 استدعاء للنماذج و 0 توكنز ما لم تتغير الواجهة)، وخادم MCP المدمج (e2e mcp) وتوليد مهارات التحقق الذاتية للمشاريع (verify-&lt;app&gt;).</t>
+        </is>
+      </c>
+      <c r="E10" s="83" t="n"/>
     </row>
     <row r="11" ht="45" customHeight="1" s="55">
       <c r="A11" s="67" t="n">
@@ -6684,19 +7087,20 @@
       </c>
       <c r="B11" s="68" t="inlineStr">
         <is>
-          <t>🛡️ درع التطهير البصري ومكافحة AI Slop (Impeccable Design Guard)</t>
+          <t>🔍 الهندسة العكسية للتطبيقات والحزم (Reverse Engineer Anything)</t>
         </is>
       </c>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>impeccable-design-guard: نفذ تدقيقاً بصرياً شاملاً للواجهة وفق بروتوكول /impeccable audit وموسوعة Component Gallery، وتحقق من تباين الألوان WCAG AA والتسلسل الهرمي.</t>
+          <t>استكشف المورد https://github.com/morluto/rea أو نفذ: npx -y rea-agents@latest</t>
         </is>
       </c>
       <c r="D11" s="70" t="inlineStr">
         <is>
-          <t>تطهير الواجهات من ركاكة الذكاء الاصطناعي (AI Slop)، موازنة التباين، ضبط التسلسل الهرمي للأزرار، والتأكد من مطابقة معايير الوصولية وتجاوب الشاشات.</t>
-        </is>
-      </c>
+          <t>وكيل الهندسة العكسية REA لتحليل الحزم الثنائية، تطبيقات Electron، حزم أندرويد APK، وتفكيك الأكواد واستخراج مسارات الـ API والمفاتيح والمخططات.</t>
+        </is>
+      </c>
+      <c r="E11" s="83" t="n"/>
     </row>
     <row r="12" ht="45" customHeight="1" s="55">
       <c r="A12" s="67" t="n">
@@ -6704,19 +7108,20 @@
       </c>
       <c r="B12" s="68" t="inlineStr">
         <is>
-          <t>🎬 محرك فيزياء الحركة وتوليد الفيديو بالكود (HyperFrames Motion Engine)</t>
+          <t>🎨 تصميم وبناء مواصفات DESIGN.md (Design MD Architect)</t>
         </is>
       </c>
       <c r="C12" s="69" t="inlineStr">
         <is>
-          <t>hyperframes-motion-engine: صمم حركات تفاعلية فائقة النعومة بمعادلات الزنبرك الطبيعي (Spring Physics) من Kinetics، أو ولد فيديو استعراضي للمنتج بالكود عبر HTML/CSS/GSAP.</t>
+          <t>design-md-architect: أنشئ ملف DESIGN.md متكامل للمشروع وفق مواصفات Google Stitch و Refero Styles مع ضبط باليت الألوان الدلالية، ومقاييس الخطوط والتباعد، وقواعد RTL.</t>
         </is>
       </c>
       <c r="D12" s="70" t="inlineStr">
         <is>
-          <t>دمج فيزياء الزنبرك الطبيعية في الواجهات (Kinetics)، وتوليد فيديوهات المنتجات والعروض التوضيحية برمجياً بالكود (HyperFrames) وفق إيقاع إعلانات وادي السيليكون (WhatShips).</t>
-        </is>
-      </c>
+          <t>توليد وتوحيد مواصفات DESIGN.md المرجعية للمشروع لضمان التماسك البصري لكافة وكلاء الذكاء الاصطناعي (Claude Code, Cursor, Codex, Gemini, Antigravity) ومنع العشوائية.</t>
+        </is>
+      </c>
+      <c r="E12" s="83" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1" s="55">
       <c r="A13" s="67" t="n">
@@ -6724,19 +7129,20 @@
       </c>
       <c r="B13" s="68" t="inlineStr">
         <is>
-          <t>🦆 جسر أبحاث Duck.ai المجاني | Duck.ai Zero-Cost Research Bridge</t>
+          <t>🛡️ درع التطهير البصري ومكافحة AI Slop (Impeccable Design Guard)</t>
         </is>
       </c>
       <c r="C13" s="69" t="inlineStr">
         <is>
-          <t>"استكشف المورد duck.ai" / "duckai bridge" / "شغل جسر duckai"</t>
+          <t>impeccable-design-guard: نفذ تدقيقاً بصرياً شاملاً للواجهة وفق بروتوكول /impeccable audit وموسوعة Component Gallery، وتحقق من تباين الألوان WCAG AA والتسلسل الهرمي.</t>
         </is>
       </c>
       <c r="D13" s="70" t="inlineStr">
         <is>
-          <t>تفعيل مهارة وجسر أبحاث Duck.ai للاستعلام المجاني من نماذج GPT-4o-mini و Claude 3 Haiku و Llama 3.3 وتوفير Sandbox لاختبارات n8n و FastMCP وحفظ كوتا النماذج التجارية لوكالة Autovem.</t>
-        </is>
-      </c>
+          <t>تطهير الواجهات من ركاكة الذكاء الاصطناعي (AI Slop)، موازنة التباين، ضبط التسلسل الهرمي للأزرار، والتأكد من مطابقة معايير الوصولية وتجاوب الشاشات.</t>
+        </is>
+      </c>
+      <c r="E13" s="83" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1" s="55">
       <c r="A14" s="67" t="n">
@@ -6744,19 +7150,20 @@
       </c>
       <c r="B14" s="68" t="inlineStr">
         <is>
-          <t>🦆 جسر أبحاث Duck.ai المجاني | Duck.ai Zero-Cost Research Bridge</t>
+          <t>🎬 محرك فيزياء الحركة وتوليد الفيديو بالكود (HyperFrames Motion Engine)</t>
         </is>
       </c>
       <c r="C14" s="69" t="inlineStr">
         <is>
-          <t>"استكشف المورد duck.ai" / "duckai bridge" / "شغل جسر duckai"</t>
+          <t>hyperframes-motion-engine: صمم حركات تفاعلية فائقة النعومة بمعادلات الزنبرك الطبيعي (Spring Physics) من Kinetics، أو ولد فيديو استعراضي للمنتج بالكود عبر HTML/CSS/GSAP.</t>
         </is>
       </c>
       <c r="D14" s="70" t="inlineStr">
         <is>
-          <t>تفعيل مهارة وجسر أبحاث Duck.ai للاستعلام المجاني من نماذج GPT-4o-mini و Claude 3 Haiku و Llama 3.3 وتوفير Sandbox لاختبارات n8n و FastMCP وحفظ كوتا النماذج التجارية لوكالة Autovem.</t>
-        </is>
-      </c>
+          <t>دمج فيزياء الزنبرك الطبيعية في الواجهات (Kinetics)، وتوليد فيديوهات المنتجات والعروض التوضيحية برمجياً بالكود (HyperFrames) وفق إيقاع إعلانات وادي السيليكون (WhatShips).</t>
+        </is>
+      </c>
+      <c r="E14" s="83" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1" s="55">
       <c r="A15" s="67" t="n">
@@ -6764,19 +7171,125 @@
       </c>
       <c r="B15" s="68" t="inlineStr">
         <is>
+          <t>🦆 جسر أبحاث Duck.ai المجاني | Duck.ai Zero-Cost Research Bridge</t>
+        </is>
+      </c>
+      <c r="C15" s="69" t="inlineStr">
+        <is>
+          <t>"استكشف المورد duck.ai" / "duckai bridge" / "شغل جسر duckai"</t>
+        </is>
+      </c>
+      <c r="D15" s="70" t="inlineStr">
+        <is>
+          <t>تفعيل مهارة وجسر أبحاث Duck.ai للاستعلام المجاني من نماذج GPT-4o-mini و Claude 3 Haiku و Llama 3.3 وتوفير Sandbox لاختبارات n8n و FastMCP وحفظ كوتا النماذج التجارية لوكالة Autovem.</t>
+        </is>
+      </c>
+      <c r="E15" s="83" t="n"/>
+    </row>
+    <row r="16" ht="45" customHeight="1" s="55">
+      <c r="A16" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="68" t="inlineStr">
+        <is>
           <t>🎬 أخصائي المونتاج والإخراج الفني بالذكاء الاصطناعي (ai-video-montage-specialist)</t>
         </is>
       </c>
-      <c r="C15" s="69" t="inlineStr">
+      <c r="C16" s="69" t="inlineStr">
         <is>
           <t>قم بتحليل فيديو العميل [البراند] واستخراج ملف الصوت والـ Contact Sheet، واستخرج التوقيتات الدقيقة بالملي ثانية عبر Whisper، ونفذ القطع الأولي (Rough Cut) بإزالة السكتات وتوليد ملف EDL، ثم طبق نظام التصميم ومكافحة النمطية في تركيبة Remotion.</t>
         </is>
       </c>
-      <c r="D15" s="70" t="inlineStr">
+      <c r="D16" s="70" t="inlineStr">
         <is>
           <t>أخصائي المونتاج والإخراج الفني الذاتي: إدارة خط إنتاج الفيديو البرمجي بالكود استناداً لهندسة غريب الشيخ؛ فحص FFmpeg واستخراج الصوت النقي 16kHz، تحليل المساحات السلبية (Negative Space) لمنع تغطية وجه المتحدث، تفريغ Whisper بالملي ثانية، توليد ملفات EDL لبريمير ودافينشي، إخراج المشاهد بأنماط Focus و Whiteboard و Screencast، ورندرة Remotion React ومكافحة ركاكة الـ AI Slop.</t>
         </is>
       </c>
+      <c r="E16" s="83" t="n"/>
+    </row>
+    <row r="17" ht="45" customHeight="1" s="55">
+      <c r="A17" s="67" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="68" t="inlineStr">
+        <is>
+          <t>🧹 تنقية الكود والتوثيق من حشو الذكاء الاصطناعي (Unslop Code &amp; English Prose Purifier)</t>
+        </is>
+      </c>
+      <c r="C17" s="69" t="inlineStr">
+        <is>
+          <t>claude -p "Review this PR diff and apply unslop: strip obvious comments and reduce boilerplate." / "/unslop" / "نظف الكود من الحشو"</t>
+        </is>
+      </c>
+      <c r="D17" s="70" t="inlineStr">
+        <is>
+          <t>مسح التعليقات التوليدية البديهية (مثل // loop over users)، وحذف التغليفات الزائدة (Over-abstraction)، وتبسيط الصياغة الإنجليزية التقنية مع الحفاظ الكامل على نصوص العربية وRTL (مستخلص من pstack / Lauren Tan).</t>
+        </is>
+      </c>
+      <c r="E17" s="83" t="n"/>
+    </row>
+    <row r="18" ht="45" customHeight="1" s="55">
+      <c r="A18" s="67" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="68" t="inlineStr">
+        <is>
+          <t>💥 تحليل نصف قطر الانفجار وتتبع التبعيات (Blast Radius Pre-Merge Verifier)</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>claude -p "What is the blast radius of changing &lt;target_function_or_file&gt;?" / "blast-radius" / "نطاق التأثير"</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="inlineStr">
+        <is>
+          <t>تحليل نصف قطر الانفجار وتتبع التبعيات العميقة عبر Git قبل دمج التعديلات (مخططات JSON، أعمدة DB، الذاكرة المؤقتة، واستدعاءات دورة الحياة)، مع إلزام الوكيل بإثبات الأمان عبر تشغيل كود تجريبي حقيقي لا مجرد افتراض.</t>
+        </is>
+      </c>
+      <c r="E18" s="83" t="n"/>
+    </row>
+    <row r="19" ht="45" customHeight="1" s="55">
+      <c r="A19" s="67" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="68" t="inlineStr">
+        <is>
+          <t>⚔️ حلبة التنافس المعماري وتطعيم الحلول (Multi-Model Architecture Arena &amp; Grafting)</t>
+        </is>
+      </c>
+      <c r="C19" s="69" t="inlineStr">
+        <is>
+          <t>claude -p "Throw the architecture problem into the arena with Candidate A (OpenCode GLM) and Candidate B (agcli Gemini), cross-judged by Claude Opus." / "/arena" / "أطلق حلبة المنافسة"</t>
+        </is>
+      </c>
+      <c r="D19" s="70" t="inlineStr">
+        <is>
+          <t>إطلاق حلبة تنافس بين مرشحين (OpenCode للمنطق و agcli للواجهات)، مع تحكيم وتطعيم الأفكار الهندسية الفضلى بواسطة Claude Code Opus Max في حل موحد متكامل.</t>
+        </is>
+      </c>
+      <c r="E19" s="83" t="n"/>
+    </row>
+    <row r="20" ht="45" customHeight="1" s="55">
+      <c r="A20" s="67" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="68" t="inlineStr">
+        <is>
+          <t>🔒 تثبيت الأخطاء البرمجية نهائياً في الاختبارات (Correct: Bug-to-CI Regression Lock)</t>
+        </is>
+      </c>
+      <c r="C20" s="69" t="inlineStr">
+        <is>
+          <t>claude -p "Apply correct: diagnose root cause and lock it into our test suite so this regression never recurs." / "/correct" / "صحح نهائياً واقفل الثغرة"</t>
+        </is>
+      </c>
+      <c r="D20" s="70" t="inlineStr">
+        <is>
+          <t>منع الاكتفاء بالترقيع المؤقت للأعطال البرمجية؛ تحويل كل خلل إلى فحص آلي دائم في اختبارات CI يفشل فوراً في حال تكرار الخلل مستقبلاً مع توثيق السبب الجذري ومحاصرته بسياج برمجي.</t>
+        </is>
+      </c>
+      <c r="E20" s="83" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6789,7 +7302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6997,6 +7510,46 @@
       <c r="D10" s="14" t="inlineStr">
         <is>
           <t>تخزين تفضيلات المستخدم العالمية والاشتراكات عبر كافة المشاريع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="72" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="73" t="inlineStr">
+        <is>
+          <t>🐍 ترقية وتثبيت بايثون الحديثة (Python 3.14/3.13) عبر uv مع حماية أوبونتو</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>curl -LsSf https://astral.sh/uv/install.sh | sh &amp;&amp; export PATH="/home/t/.local/bin:/home/t/.local/bin:/home/t/.gemini/antigravity/bin:/usr/local/sbin:/usr/local/bin:/usr/sbin:/usr/bin:/sbin:/bin:/usr/games:/usr/local/games:/usr/lib/wsl/lib:/mnt/c/Users/Kt/AppData/Roaming/Antigravity/bin:/mnt/c/Program Files/Eclipse Adoptium/jdk-17.0.19.10-hotspot/bin:/mnt/c/WINDOWS/system32:/mnt/c/WINDOWS:/mnt/c/WINDOWS/System32/Wbem:/mnt/c/WINDOWS/System32/WindowsPowerShell/v1.0/:/mnt/c/WINDOWS/System32/OpenSSH/:/mnt/c/Program Files/Common Files/Autodesk Shared/:/mnt/c/Program Files/Microsoft SQL Server/150/Tools/Binn/:/mnt/c/Program Files/dotnet/:/mnt/c/Program Files (x86)/Microsoft SQL Server/160/Tools/Binn/:/mnt/c/Program Files/Microsoft SQL Server/160/Tools/Binn/:/mnt/c/Program Files/Microsoft SQL Server/Client SDK/ODBC/170/Tools/Binn/:/mnt/c/Program Files/Microsoft SQL Server/160/DTS/Binn/:/mnt/c/Program Files/NVIDIA Corporation/NVIDIA App/NvDLISR:/mnt/c/Program Files (x86)/NVIDIA Corporation/PhysX/Common:/mnt/c/Program Files/nodejs/:/mnt/c/Program Files/Docker/Docker/resources/bin:/mnt/c/Program Files/Git/cmd:/mnt/f/AI PROJECTS/flutter/bin:/mnt/c/Program Files/GitHub CLI/:/mnt/c/Program Files/PowerShell/7/:/mnt/c/Users/Kt/.kimi-code/bin:/mnt/c/Users/Kt/.cargo/bin:/mnt/c/Users/Kt/AppData/Local/Programs/Python/Python314/Scripts/:/mnt/c/Users/Kt/AppData/Local/Programs/Python/Python314/:/mnt/c/Users/Kt/AppData/Local/Microsoft/WindowsApps:/mnt/c/Users/Kt/AppData/Roaming/npm:/mnt/c/Users/Kt/AppData/Local/Programs/Microsoft VS Code/bin:/mnt/c/Users/Kt/AppData/AndroidCLI:/mnt/c/Users/Kt/AppData/Local/Programs/Antigravity IDE/bin:/mnt/c/Users/Kt/AppData/Local/Programs/Antigravity IDE00/bin:/mnt/c/Users/Kt/AppData/Local/Programs/Ollama:/mnt/f/flutter/bin" &amp;&amp; uv python install 3.14 3.13 &amp;&amp; ln -sf /home/t/.local/share/uv/python/cpython-3.14-linux-x86_64-gnu/bin/python3.14 ~/.local/bin/python3.14 &amp;&amp; ln -sf /home/t/.local/share/uv/python/cpython-3.13-linux-x86_64-gnu/bin/python3.13 ~/.local/bin/python3.13</t>
+        </is>
+      </c>
+      <c r="D11" s="73" t="inlineStr">
+        <is>
+          <t>تثبيت وتفعيل أحدث نسخ بايثون الرسمية (Python 3.14.7 و 3.13.15) في بيئة أوبونتو WSL2 دون المساس بإصدار بايثون النظامي (3.12) لحماية أدوات apt، وتفعيل مدير الحزم فائق السرعة uv لإنشاء البيئات اللحظية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="72" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="73" t="inlineStr">
+        <is>
+          <t>🚀 ترحيل مشاريع ويندوز إلى نظام أوبونتو الداخلي (ext4) وتسريع I/O بمقدار 20 ضعفاً</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>mkdir -p ~/projects &amp;&amp; rsync -avh --info=progress2 "/mnt/&lt;drive&gt;/&lt;path&gt;" ~/projects/ &amp;&amp; cd ~/projects/&lt;project_name&gt; &amp;&amp; git config core.autocrlf input</t>
+        </is>
+      </c>
+      <c r="D12" s="73" t="inlineStr">
+        <is>
+          <t>نقل مشاريع البرمجة والذكاء الاصطناعي من مسارات أقراص ويندوز البطيئة (/mnt/...) إلى نظام ملفات لينكس الأصلي ext4 لتسريع فحص Git وبناء الحزم بمقدار 10-20 ضعفاً وتفادي تحذيرات المحرر، مع التنظيف المسبق لمنع امتلاء قرص C.</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -7373,6 +7926,26 @@
       <c r="D15" s="70" t="inlineStr">
         <is>
           <t>أمر هندسي لتوليد عرض سعر ومقايسة غير مسعرة لأعمال الدرابزينات الزجاجية (94 م2 ممرات بقطاع يو تشانيل أسود 8 سم + 106 م2 أدراج بأرجل سبايدر 16 سم سوداء = إجمالي 200 م2) لصالح مؤسسة تل العمارة للمقاولات على الورق الرسمي لمصنع منصة الإبداع للمعادن (XLSX + DOCX + PDF) بقيد الصفحة الواحدة الصارم.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1" s="55">
+      <c r="A16" s="67" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="68" t="inlineStr">
+        <is>
+          <t>📑 حوكمة وتوليد عروض أسعار مصنع الإبداع بالترقيم التسلسلي الآلي</t>
+        </is>
+      </c>
+      <c r="C16" s="69" t="inlineStr">
+        <is>
+          <t>بصفتك مهندس التسعير والعقود والحوكمة بمصنع منصة الإبداع للمعادن، اعتمد المسار المركزي [G:\M.Yonis\03_المشاريع\مشاريع_أخرى_وعملاء\مصنع_الابداع\Clients] لإدارة كافة عروض الأسعار والمقايسات. التزم بالبروتوكول التالي: 1) فحص المجلد وسجل الفهرسة المركزي [QUOTATION_LEDGER.xlsx] لاكتشاف أعلى رقم تسلسلي وتخصيص الرقم التالي تلقائياً بنمط [MAF-YYYY-NN] أو [MAF-CLI-YYYY-NN]. 2) إنشاء مجلد فرعي مستقل لكل عميل بالنمط [[الرقم_التسلسلي]_[اسم_العميل]_[المشروع]]. 3) توليد الحزمة الثلاثية المعتمدة (XLSX بمعادلات ديناميكية، DOCX بمعمارية BiDi، و PDF بالورق الرسمي 300 DPI للمصنع وقيد الصفحة الواحدة و0 أرقام هندية مشرقية). 4) تحديث السجل المركزي آلياً وتوليد روابط ويندوز المباشرة file:///G:/...</t>
+        </is>
+      </c>
+      <c r="D16" s="70" t="inlineStr">
+        <is>
+          <t>حوكمة مركزية لإنتاج وأرشفة عروض أسعار ومقايسات مصنع منصة الإبداع للمعادن مع الفحص الآلي للترقيم التسلسلي التالي، إنشاء مجلدات العملاء، تحديث سجل الفهرسة المركزي، وتصدير الحزمة الثلاثية المعتمدة.</t>
         </is>
       </c>
     </row>
@@ -7475,7 +8048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -7506,27 +8079,26 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="68" t="inlineStr">
         <is>
           <t>📂 إظهار الملفات في مستكشف ويندوز وتصديرها لسطح المكتب (Reveal &amp; Desktop Hub - C-81)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="69" t="inlineStr">
         <is>
           <t>reveal "&lt;Full_Path&gt;"</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="70" t="inlineStr">
         <is>
           <t>المعيار الإلزامي [C-81] لأدوات ومستندات Antigravity: يقوم بترجمة مسارات WSL إلى ويندوز، نسخ الملف فوراً إلى مجلد المستندات_المولدة على سطح المكتب (C:\Users\Kt\Desktop\المستندات_المولدة\)، وفتح مستكشف الملفات مع تظليل الملف تلقائياً وبشكل غير تزامني.</t>
         </is>
       </c>
+      <c r="E2" s="83" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7539,13 +8111,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
-    <col width="32" customWidth="1" style="55" min="2" max="2"/>
-    <col width="52" customWidth="1" style="55" min="3" max="3"/>
-    <col width="75" customWidth="1" style="55" min="4" max="4"/>
+    <col width="35" customWidth="1" style="55" min="2" max="2"/>
+    <col width="75" customWidth="1" style="55" min="3" max="3"/>
+    <col width="45" customWidth="1" style="55" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="55">
@@ -7567,6 +8139,128 @@
       <c r="D1" s="71" t="inlineStr">
         <is>
           <t>الوصف والاستخدام (Description &amp; Notes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1" s="55">
+      <c r="A2" s="67" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="68" t="inlineStr">
+        <is>
+          <t>📦🧹 تطهير حزم تسليم تطبيقات الويب وحيادية الفلترة (Pure Web App Bundle)</t>
+        </is>
+      </c>
+      <c r="C2" s="69" t="inlineStr">
+        <is>
+          <t># Autonomous Web Delivery Bundle Purge &amp; Filter Neutrality Invariant [C-87]
+1. Purge all PDF reports, Word files, internal markdown notes, and raw reference Excel files from client delivery bundle (.zip).
+2. Restrict bundle exclusively to runtime essentials: active app HTML, blank template HTML, offline vendor scripts (xlsx.full.min.js, pdf.min.js, pdf.worker.js), and brand assets. Target size: &lt; 1 MB.
+3. Enforce Filter Neutrality: remove hardcoded past month chips, default initial view to Full Period, and compute counters dynamically from active dataset.</t>
+        </is>
+      </c>
+      <c r="D2" s="70" t="inlineStr">
+        <is>
+          <t>معيار تطهير حزم تسليم تطبيقات الويب المستقلة (SPAs) ولوحات التحليلات للعملاء (المعيار C-87 و Rule 60). حصر الحزمة في ملفات تشغيل الويب فقط لتقليص الحجم لأقل من 1 ميجابايت، وترسيخ حيادية الفلترة الافتراضية على كامل الفترة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="80" t="inlineStr">
+        <is>
+          <t>🎓✨ تطبيق الورشة الختامية التفاعلية للمستوى الأول (ESL Level 1 Final Review: Phonics, Senses &amp; Grammar Interactive App)</t>
+        </is>
+      </c>
+      <c r="C3" s="81" t="inlineStr">
+        <is>
+          <t># 🎓 Master Educational Prompt: Level 1 Young Learners Final Revision Interactive App
+## 🎯 Target Audience &amp; Core Objective
+- **Learners:** Young ESL beginners (Level 1 / Kindergarten / Grade 1).
+- **Format:** High-engagement, standalone interactive single-page web app / teaching dashboard.
+- **Key Pedagogical Pillars:** Demonstratives, Senses + Body Parts (3-Sentence Triad), Indefinite Articles (a vs an), and CVC Word Families (Short a &amp; Short e).
+---
+## 🛠️ Module Architecture &amp; Functional Specifications
+### 1. Visual &amp; Zoom Architecture (UI/UX)
+- Every concept must be illustrated with a colorful, friendly, child-appropriate vector graphic or image.
+- **Interactive Image Zoom Feature:** Clicking any image opens a high-definition Lightbox modal with interactive Zoom In (+), Zoom Out (-), Reset, and Pan controls for detailed classroom presentation on smartboards.
+### 2. Demonstratives &amp; Quantity Warm-Up
+- **This is** (Singular: 1 object/organ) vs. **These are** (Plural: 2 objects/organs).
+- Integration of `have`: "I have one..." vs. "I have two...".
+### 3. Body Parts &amp; 5 Senses Integration (The 3-Sentence Triad)
+Each organ must follow this exact 3-sentence cumulative sentence pattern:
+1. **Eyes:**
+   - Sentence 1: "These are my eyes."
+   - Sentence 2: "I have two eyes."
+   - Sentence 3: "I can see with my eyes."
+2. **Nose:**
+   - Sentence 1: "This is my nose."
+   - Sentence 2: "I have one nose."
+   - Sentence 3: "I can smell with my nose."
+3. **Ears:**
+   - Sentence 1: "These are my ears."
+   - Sentence 2: "I have two ears."
+   - Sentence 3: "I can hear with my ears."
+4. **Tongue:**
+   - Sentence 1: "This is my tongue."
+   - Sentence 2: "I have one tongue."
+   - Sentence 3: "I can taste with my tongue."
+5. **Mouth:**
+   - Sentence 1: "This is my mouth."
+   - Sentence 2: "I have one mouth."
+   - Sentence 3: "I can eat / speak with my mouth."
+6. **Hands:**
+   - Sentence 1: "These are my hands."
+   - Sentence 2: "I have two hands."
+   - Sentence 3: "I can touch with my hands."
+### 4. Indefinite Articles Module: `a` vs. `an`
+- Visual anchor: `a` before consonant sounds; `an` before vowel sounds (a, e, i, o, u).
+- **5 Examples for 'a':** a cat, a dog, a car, a book, a hat.
+- **5 Examples for 'an':** an apple, an elephant, an insect, an orange, an umbrella.
+- Interactive sorting basket game for students to drag or click items into Basket `a` or Basket `an`.
+### 5. CVC Phonics Word Families Soundboard (Short a &amp; Short e)
+- **Short `a` (/æ/) Word Families (10 Words):**
+  - Family `-at` (5 words): cat, bat, hat, mat, rat.
+  - Family `-an` (5 words): can, fan, man, pan, van.
+- **Short `e` (/ɛ/) Word Families (10 Words):**
+  - Family `-en` (5 words): hen, pen, ten, men, den.
+  - Family `-et` (5 words): net, pet, wet, jet, vet.
+  *(Note: Replaced spoken phonetic slip 'pin/tin' which belong to Short 'i' (/ɪ/) to avoid phonemic confusion for young learners).*
+- Interactive blend soundboard: Click individual sounds (/k/ + /æt/ -&gt; cat).
+### 6. Audio Pronunciation &amp; Gamification
+- Built-in Web Speech API Text-to-Speech: Clicking any word or sentence plays natural, clear English pronunciation.
+- Gamified Review Quiz with instant audio feedback (synthesized Web Audio beeps/chimes) and star rewards.</t>
+        </is>
+      </c>
+      <c r="D3" s="82" t="inlineStr">
+        <is>
+          <t>موجه هندسي بيداغوجي متكامل لإنتاج تطبيق ومراجعة تفاعلية للمستوى الأول لتعليم اللغة الإنجليزية للأطفال (Level 1 ESL). يدمج قواعد الإشارة (This is/These are)، والحواس الخمس عبر نموذج الجمل الثلاث المتراكمة (Demonstrative + Have + Sense Verb)، وأدوات التنكير (a/an)، وعائلات كلمات الـ CVC للـ Short A و Short E مع تصحيح الانزلاقات الصوتية في التسجيل الشفوي للمعلمة، وتوفير خاصية تقريب الصور (Zoom in/out) ونطق صوتي تفاعلي Web Speech API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="55">
+      <c r="A4" s="67" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="68" t="inlineStr">
+        <is>
+          <t>📊 تقرير إنجاز الميزات للعميل الإداري (Executive Client Report)</t>
+        </is>
+      </c>
+      <c r="C4" s="69" t="inlineStr">
+        <is>
+          <t>قم بإعداد تقرير تنفيذي رسمي بصيغة PDF يوثق الميزات الـ 6 المنجزة حديثاً لتقديمها للعميل الإداري، مع مراعاة الضوابط التالية:
+1. صياغة غير تقنية 100%: حظر أي مصطلحات برمجية أو هندسية (API, DB, Docker, Endpoints).
+2. هيكل ثلاثي مبسط لكل ميزة: (ما هي الميزة؟ كيف تفيدك وتفيد المركز؟ كيف تستخدمها في خطوتين بسيطتين؟).
+3. أرقام إنجليزية (0-9) وهوية بصرية رسمية متناسقة بخط Cairo وبطاقات ملونة واضحة.
+4. نشر التقرير برابط HTTPS مباشر ومشفر من الخادم للمعاينة الفورية من الجوال، وحفظ نسخة PDF محلية.</t>
+        </is>
+      </c>
+      <c r="D4" s="70" t="inlineStr">
+        <is>
+          <t>موجه مهندس لإعداد ونشر تقارير الميزات والمنجزات للعملاء غير التقنيين طبقاً للمعيار [C-99]، يضمن إيصال القيمة الإدارية والمالية وتبسيط طريقة الاستخدام دون تعقيد تقني.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(prompt-library): add OpenCode Go fleet quota maximizer and Claude consultation commands (Hook 26)
</commit_message>
<xml_diff>
--- a/مكتبة الأوامر.xlsx
+++ b/مكتبة الأوامر.xlsx
@@ -5061,7 +5061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="29" min="1" max="1"/>
@@ -5949,6 +5949,26 @@
       </c>
       <c r="E36" s="83" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="67" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="68" t="inlineStr">
+        <is>
+          <t>🧠 استشارة وتحكيم كلود المعماري المباشر للأسطول (Claude Headless Architectural Consultation &amp; Audit)</t>
+        </is>
+      </c>
+      <c r="C37" s="69" t="inlineStr">
+        <is>
+          <t>cmd.exe /c "cd /d F:\AI PROJECTS\Autovemtech &amp;&amp; claude -p - &lt; scripts/claude_consultation_prompt.txt"</t>
+        </is>
+      </c>
+      <c r="D37" s="70" t="inlineStr">
+        <is>
+          <t>تشغيل استدعاء استشاري مباشر في الخلفية لـ Claude Code CLI (Opus Max) تحت القيد [C-25] و [C-91] لتحكيم القرارات المعمارية الحساسة، فحص الثغرات (Devil's Advocate Audit)، وإصدار توجيهات الأسطول لحرق كوتا OpenCode Go واستغلالها دون استنزاف سياق واجهة المستخدم وبلا نسخ يدوي.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3"/>
@@ -5961,7 +5981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6409,6 +6429,46 @@
         </is>
       </c>
       <c r="E19" s="83" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="67" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="68" t="inlineStr">
+        <is>
+          <t>🧠 استشارة وتحكيم كلود المعماري المباشر للأسطول (Claude Headless Architectural Consultation &amp; Audit)</t>
+        </is>
+      </c>
+      <c r="C20" s="69" t="inlineStr">
+        <is>
+          <t>cmd.exe /c "cd /d F:\AI PROJECTS\Autovemtech &amp;&amp; claude -p - &lt; scripts/claude_consultation_prompt.txt"</t>
+        </is>
+      </c>
+      <c r="D20" s="70" t="inlineStr">
+        <is>
+          <t>تشغيل استدعاء استشاري مباشر في الخلفية لـ Claude Code CLI (Opus Max) تحت القيد [C-25] و [C-91] لتحكيم القرارات المعمارية الحساسة، فحص الثغرات (Devil's Advocate Audit)، وإصدار توجيهات الأسطول لحرق كوتا OpenCode Go واستغلالها دون استنزاف سياق واجهة المستخدم وبلا نسخ يدوي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="67" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="68" t="inlineStr">
+        <is>
+          <t>⚡ مفوض واستهلاك كوتا OpenCode Go الموحد للأسطول (OpenCode Go Fleet Quota Maximizer &amp; Dispatcher)</t>
+        </is>
+      </c>
+      <c r="C21" s="69" t="inlineStr">
+        <is>
+          <t>python tools/opencode_dispatcher.py --task "&lt;task_instructions&gt;" --model glm</t>
+        </is>
+      </c>
+      <c r="D21" s="70" t="inlineStr">
+        <is>
+          <t>أداة التفويض المركزية لأسطول Autovemtech لحرق كوتا اشتراك OpenCode Go ($10 شهرياً) بالكامل، عبر إلقاء مهام كتابة البويلربليت، ترحيل قواعد البيانات، والمسائل الخوارزمية البديلة لكودكس على نماذج OpenCode Go الأربعة (GLM Flash, DeepSeek V4.1, Muse Spark, MiniMax) مع تسجيل السجلات في fleet_orders وتطبيق القيد [C-78] لحماية تدفق البث.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8048,7 +8108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -8099,6 +8159,26 @@
         </is>
       </c>
       <c r="E2" s="83" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="67" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="68" t="inlineStr">
+        <is>
+          <t>⚡ مفوض واستهلاك كوتا OpenCode Go الموحد للأسطول (OpenCode Go Fleet Quota Maximizer &amp; Dispatcher)</t>
+        </is>
+      </c>
+      <c r="C3" s="69" t="inlineStr">
+        <is>
+          <t>python tools/opencode_dispatcher.py --task "&lt;task_instructions&gt;" --model glm</t>
+        </is>
+      </c>
+      <c r="D3" s="70" t="inlineStr">
+        <is>
+          <t>أداة التفويض المركزية لأسطول Autovemtech لحرق كوتا اشتراك OpenCode Go ($10 شهرياً) بالكامل، عبر إلقاء مهام كتابة البويلربليت، ترحيل قواعد البيانات، والمسائل الخوارزمية البديلة لكودكس على نماذج OpenCode Go الأربعة (GLM Flash, DeepSeek V4.1, Muse Spark, MiniMax) مع تسجيل السجلات في fleet_orders وتطبيق القيد [C-78] لحماية تدفق البث.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(governance): add [C-105] design resources standard, update Hook 31 triggers, and curate prompt library
</commit_message>
<xml_diff>
--- a/مكتبة الأوامر.xlsx
+++ b/مكتبة الأوامر.xlsx
@@ -48,7 +48,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="34">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -242,6 +242,22 @@
       <name val="Consolas"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001B365D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000F172A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -287,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -575,11 +591,25 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -800,6 +830,18 @@
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5981,7 +6023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -6467,6 +6509,26 @@
       <c r="D21" s="70" t="inlineStr">
         <is>
           <t>أداة التفويض المركزية لأسطول Autovemtech لحرق كوتا اشتراك OpenCode Go ($10 شهرياً) بالكامل، عبر إلقاء مهام كتابة البويلربليت، ترحيل قواعد البيانات، والمسائل الخوارزمية البديلة لكودكس على نماذج OpenCode Go الأربعة (GLM Flash, DeepSeek V4.1, Muse Spark, MiniMax) مع تسجيل السجلات في fleet_orders وتطبيق القيد [C-78] لحماية تدفق البث.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1" s="55">
+      <c r="A22" s="67" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="68" t="inlineStr">
+        <is>
+          <t>🎨🏛️ خطاف معاينة وتنسيق العمل الجماعي لمراجع التصميم (Design Resources Fleet Teamwork Orchestrator - Hook 31)</t>
+        </is>
+      </c>
+      <c r="C22" s="69" t="inlineStr">
+        <is>
+          <t>python3 tools/fleet_teamwork_orchestrator.py -w .agents/fleet_teamwork_design_vault status / "الخطاف 31 استكشف الموارد" / "معاينة العمل الجماعي للأسطول"</t>
+        </is>
+      </c>
+      <c r="D22" s="70" t="inlineStr">
+        <is>
+          <t>تفعيل فريق عمل الأسطول الموزع (Hook 31) لاستكشاف، تحليل، وتكامل مراجع التصميم الـ 8 وتوثيق أدلة التسليم الفيزيائية في handoff.md واعتمادها حصرياً بواسطة Claude Code CLI.</t>
         </is>
       </c>
     </row>
@@ -6907,7 +6969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -7350,6 +7412,46 @@
         </is>
       </c>
       <c r="E20" s="83" t="n"/>
+    </row>
+    <row r="21" ht="45" customHeight="1" s="55">
+      <c r="A21" s="67" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="68" t="inlineStr">
+        <is>
+          <t>🌐 أداة تصفح الوكلاء الذاتي Webcmd (Webcmd Agent Browser)</t>
+        </is>
+      </c>
+      <c r="C21" s="69" t="inlineStr">
+        <is>
+          <t>webcmd --profile default session create "AgentTask" &amp;&amp; webcmd --session &lt;session-id&gt; browser snapshot --snapshot-mode act</t>
+        </is>
+      </c>
+      <c r="D21" s="70" t="inlineStr">
+        <is>
+          <t>تفعيل متصفح الوكلاء ذاتي التعلم (Webcmd) لتنفيذ مهام التصفح التفاعلي، فحص واجهات الهبوط، واستخراج البيانات بذاكرة Sitemap تلقائية توفر حتى 90% من التوكنز مع محرك CloakBrowser للتخفي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1" s="55">
+      <c r="A22" s="67" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="68" t="inlineStr">
+        <is>
+          <t>🎨🏛️ مستودع مراجع التصميم العالمية وهندسة الواجهات (Design Resources Master Vault - 8 Sites)</t>
+        </is>
+      </c>
+      <c r="C22" s="69" t="inlineStr">
+        <is>
+          <t>Skill(superpowers:design-vault) / "استكشف مراجع التصميم" / "مستودع مراجع التصميم" / "design vault" / "jiro bento 60fps"</t>
+        </is>
+      </c>
+      <c r="D22" s="70" t="inlineStr">
+        <is>
+          <t>استدعاء مستودع مراجع التصميم الـ 8 المعتمدة (jiro.build لأوامر AI، navbar.gallery للقوائم، footer.design للتذييلات، cta.gallery لدعوات الإجراء، 404s.design لصفحات الخطأ، unsection.com للكتل الجاهزة، bentogrids.com لشبكات البنتو، 60fps.design للحركات السلسة) لدعم الواجهات العربية RTL وتطبيقات الويب والهواتف.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7642,7 +7744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" style="55" min="1" max="1"/>
@@ -8006,6 +8108,31 @@
       <c r="D16" s="70" t="inlineStr">
         <is>
           <t>حوكمة مركزية لإنتاج وأرشفة عروض أسعار ومقايسات مصنع منصة الإبداع للمعادن مع الفحص الآلي للترقيم التسلسلي التالي، إنشاء مجلدات العملاء، تحديث سجل الفهرسة المركزي، وتصدير الحزمة الثلاثية المعتمدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="95" customHeight="1" s="55">
+      <c r="A17" s="84" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="85" t="inlineStr">
+        <is>
+          <t>⏱️ معيار الحظر التلقائي لمدد التنفيذ في عروض الأسعار (Strict Zero-Default Duration Standard)</t>
+        </is>
+      </c>
+      <c r="C17" s="86" t="inlineStr">
+        <is>
+          <t>قاعدة تعاقدية إلزامية [Strict Zero-Default Duration]:
+يُحظر تماماً وبشكل قاطع إدراج أو افتراض أي "مدة تنفيذ" أو "مدة توريد وتركيب" في عروض الأسعار والمقايسات الصادرة لمؤسسة إعمار الفرعة أو مصنع منصة الإبداع، ما لم يطلب المستخدم أو تنص المتطلبات صراحة على تحديد مدة معينة.
+عند عدم طلب مدة التنفيذ:
+1. تُحذف خانة "مدة التنفيذ" كلياً من صناديق البيانات التعريفية في (XLSX, DOCX, PDF).
+2. يُدمج صف "موضوع العرض" بكامل العرض (Full Width Merge) لضمان التناسق البصري التام.
+3. يُحظر ذكر أي مدد زمنية في الشروط والأحكام ما عدا مدة سريان العرض التعاقدية (30 يوماً).</t>
+        </is>
+      </c>
+      <c r="D17" s="87" t="inlineStr">
+        <is>
+          <t>قيد تعاقدي وهندسي صارم لحماية المقاول قانونياً من الالتزامات الزمنية التقديرية غير المدروسة في العروض التنافسية. يلزم الوكلاء بعدم تضمين مدة التنفيذ تلقائياً إلا بتوجيه صريح، وإعادة موازنة صناديق التعريف بدمج خانة موضوع العرض عبر العرض الكامل.</t>
         </is>
       </c>
     </row>

</xml_diff>